<commit_message>
Plot the round v4.8 (Gladius+ZEPHON)
</commit_message>
<xml_diff>
--- a/assets/ledger.xlsx
+++ b/assets/ledger.xlsx
@@ -6,14 +6,14 @@
     <sheet state="visible" name="ledger" sheetId="1" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">ledger!$A$7:$P$51</definedName>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">ledger!$A$7:$P$53</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="134">
   <si>
     <t>Civ-likeness Rating System</t>
   </si>
@@ -287,6 +287,12 @@
     <t>25.5/6.5</t>
   </si>
   <si>
+    <t>ZEPHON (2024–current, 1.3)</t>
+  </si>
+  <si>
+    <t>25.0/7.0</t>
+  </si>
+  <si>
     <t>Age of Wonders 3 (2014)</t>
   </si>
   <si>
@@ -306,6 +312,12 @@
   </si>
   <si>
     <t>21.5/8.5</t>
+  </si>
+  <si>
+    <t>Warhammer 40,000: Gladius (2018–26, 11 factions)</t>
+  </si>
+  <si>
+    <t>24.0/5.5</t>
   </si>
   <si>
     <t>Total War: Warhammer III (2022, IE + 9.0)</t>
@@ -1118,7 +1130,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="38.0"/>
+    <col customWidth="1" min="1" max="1" width="39.13"/>
     <col customWidth="1" min="2" max="9" width="20.13"/>
     <col customWidth="1" min="10" max="10" width="28.88"/>
     <col customWidth="1" min="11" max="12" width="11.38"/>
@@ -1466,7 +1478,7 @@
         <v>40.0</v>
       </c>
       <c r="M8" s="52">
-        <f t="shared" ref="M8:M51" si="1">L8/40</f>
+        <f t="shared" ref="M8:M53" si="1">L8/40</f>
         <v>1</v>
       </c>
       <c r="N8" s="53" t="s">
@@ -2600,25 +2612,25 @@
         <v>90</v>
       </c>
       <c r="B32" s="48">
-        <v>4.5</v>
+        <v>4.0</v>
       </c>
       <c r="C32" s="48">
         <v>4.0</v>
       </c>
       <c r="D32" s="48">
+        <v>4.5</v>
+      </c>
+      <c r="E32" s="48">
         <v>4.0</v>
-      </c>
-      <c r="E32" s="48">
-        <v>3.5</v>
       </c>
       <c r="F32" s="48">
         <v>4.0</v>
       </c>
       <c r="G32" s="48">
-        <v>4.0</v>
+        <v>4.5</v>
       </c>
       <c r="H32" s="48">
-        <v>3.5</v>
+        <v>3.0</v>
       </c>
       <c r="I32" s="48">
         <v>4.0</v>
@@ -2627,22 +2639,17 @@
         <v>91</v>
       </c>
       <c r="K32" s="50">
-        <v>31.5</v>
+        <v>32.0</v>
       </c>
       <c r="L32" s="51">
-        <v>31.5</v>
+        <v>31.75</v>
       </c>
       <c r="M32" s="52">
         <f t="shared" si="1"/>
-        <v>0.7875</v>
-      </c>
-      <c r="N32" s="53" t="s">
-        <v>87</v>
-      </c>
-      <c r="P32" s="54" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K32,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
-        <v/>
-      </c>
+        <v>0.79375</v>
+      </c>
+      <c r="N32" s="53"/>
+      <c r="P32" s="54"/>
     </row>
     <row r="33">
       <c r="A33" s="47" t="s">
@@ -2652,7 +2659,7 @@
         <v>4.5</v>
       </c>
       <c r="C33" s="48">
-        <v>3.5</v>
+        <v>4.0</v>
       </c>
       <c r="D33" s="48">
         <v>4.0</v>
@@ -2667,7 +2674,7 @@
         <v>4.0</v>
       </c>
       <c r="H33" s="48">
-        <v>3.0</v>
+        <v>3.5</v>
       </c>
       <c r="I33" s="48">
         <v>4.0</v>
@@ -2676,14 +2683,14 @@
         <v>93</v>
       </c>
       <c r="K33" s="50">
-        <v>30.5</v>
+        <v>31.5</v>
       </c>
       <c r="L33" s="51">
-        <v>30.5</v>
+        <v>31.5</v>
       </c>
       <c r="M33" s="52">
         <f t="shared" si="1"/>
-        <v>0.7625</v>
+        <v>0.7875</v>
       </c>
       <c r="N33" s="53" t="s">
         <v>87</v>
@@ -2698,41 +2705,41 @@
         <v>94</v>
       </c>
       <c r="B34" s="48">
-        <v>5.0</v>
+        <v>4.5</v>
       </c>
       <c r="C34" s="48">
-        <v>3.0</v>
+        <v>3.5</v>
       </c>
       <c r="D34" s="48">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="E34" s="48">
+        <v>3.5</v>
+      </c>
+      <c r="F34" s="48">
         <v>4.0</v>
-      </c>
-      <c r="F34" s="48">
-        <v>3.5</v>
       </c>
       <c r="G34" s="48">
         <v>4.0</v>
       </c>
       <c r="H34" s="48">
-        <v>3.5</v>
+        <v>3.0</v>
       </c>
       <c r="I34" s="48">
-        <v>4.5</v>
+        <v>4.0</v>
       </c>
       <c r="J34" s="49" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="K34" s="50">
         <v>30.5</v>
       </c>
       <c r="L34" s="51">
-        <v>30.25</v>
+        <v>30.5</v>
       </c>
       <c r="M34" s="52">
         <f t="shared" si="1"/>
-        <v>0.75625</v>
+        <v>0.7625</v>
       </c>
       <c r="N34" s="53" t="s">
         <v>87</v>
@@ -2744,10 +2751,10 @@
     </row>
     <row r="35">
       <c r="A35" s="47" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B35" s="48">
-        <v>3.5</v>
+        <v>5.0</v>
       </c>
       <c r="C35" s="48">
         <v>3.0</v>
@@ -2756,35 +2763,35 @@
         <v>3.0</v>
       </c>
       <c r="E35" s="48">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="F35" s="48">
-        <v>5.0</v>
+        <v>3.5</v>
       </c>
       <c r="G35" s="48">
-        <v>5.0</v>
+        <v>4.0</v>
       </c>
       <c r="H35" s="48">
         <v>3.5</v>
       </c>
       <c r="I35" s="48">
-        <v>4.0</v>
+        <v>4.5</v>
       </c>
       <c r="J35" s="49" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K35" s="50">
-        <v>30.0</v>
+        <v>30.5</v>
       </c>
       <c r="L35" s="51">
-        <v>29.75</v>
+        <v>30.25</v>
       </c>
       <c r="M35" s="52">
         <f t="shared" si="1"/>
-        <v>0.74375</v>
+        <v>0.75625</v>
       </c>
       <c r="N35" s="53" t="s">
-        <v>45</v>
+        <v>87</v>
       </c>
       <c r="P35" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K35,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -2796,44 +2803,44 @@
         <v>97</v>
       </c>
       <c r="B36" s="48">
-        <v>4.5</v>
+        <v>3.5</v>
       </c>
       <c r="C36" s="48">
         <v>3.0</v>
       </c>
       <c r="D36" s="48">
-        <v>2.5</v>
+        <v>3.0</v>
       </c>
       <c r="E36" s="48">
-        <v>2.5</v>
+        <v>3.0</v>
       </c>
       <c r="F36" s="48">
+        <v>5.0</v>
+      </c>
+      <c r="G36" s="48">
+        <v>5.0</v>
+      </c>
+      <c r="H36" s="48">
         <v>3.5</v>
       </c>
-      <c r="G36" s="48">
-        <v>4.5</v>
-      </c>
-      <c r="H36" s="48">
-        <v>3.0</v>
-      </c>
       <c r="I36" s="48">
-        <v>3.5</v>
+        <v>4.0</v>
       </c>
       <c r="J36" s="49" t="s">
         <v>98</v>
       </c>
       <c r="K36" s="50">
-        <v>27.0</v>
+        <v>30.0</v>
       </c>
       <c r="L36" s="51">
-        <v>26.75</v>
+        <v>29.75</v>
       </c>
       <c r="M36" s="52">
         <f t="shared" si="1"/>
-        <v>0.66875</v>
+        <v>0.74375</v>
       </c>
       <c r="N36" s="53" t="s">
-        <v>87</v>
+        <v>45</v>
       </c>
       <c r="P36" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K36,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -2845,25 +2852,25 @@
         <v>99</v>
       </c>
       <c r="B37" s="48">
+        <v>4.0</v>
+      </c>
+      <c r="C37" s="48">
+        <v>4.0</v>
+      </c>
+      <c r="D37" s="48">
+        <v>4.0</v>
+      </c>
+      <c r="E37" s="48">
         <v>3.5</v>
       </c>
-      <c r="C37" s="48">
+      <c r="F37" s="48">
         <v>3.0</v>
       </c>
-      <c r="D37" s="48">
+      <c r="G37" s="48">
+        <v>4.5</v>
+      </c>
+      <c r="H37" s="48">
         <v>2.5</v>
-      </c>
-      <c r="E37" s="48">
-        <v>3.0</v>
-      </c>
-      <c r="F37" s="48">
-        <v>4.5</v>
-      </c>
-      <c r="G37" s="48">
-        <v>3.0</v>
-      </c>
-      <c r="H37" s="48">
-        <v>3.5</v>
       </c>
       <c r="I37" s="48">
         <v>4.0</v>
@@ -2872,66 +2879,61 @@
         <v>100</v>
       </c>
       <c r="K37" s="50">
-        <v>27.0</v>
+        <v>29.5</v>
       </c>
       <c r="L37" s="51">
-        <v>26.5</v>
+        <v>29.25</v>
       </c>
       <c r="M37" s="52">
         <f t="shared" si="1"/>
-        <v>0.6625</v>
-      </c>
-      <c r="N37" s="53" t="s">
-        <v>63</v>
-      </c>
-      <c r="P37" s="54" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K37,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
-        <v/>
-      </c>
+        <v>0.73125</v>
+      </c>
+      <c r="N37" s="53"/>
+      <c r="P37" s="54"/>
     </row>
     <row r="38">
-      <c r="A38" s="57" t="s">
+      <c r="A38" s="47" t="s">
         <v>101</v>
       </c>
       <c r="B38" s="48">
         <v>4.5</v>
       </c>
       <c r="C38" s="48">
-        <v>3.5</v>
+        <v>3.0</v>
       </c>
       <c r="D38" s="48">
-        <v>4.0</v>
+        <v>2.5</v>
       </c>
       <c r="E38" s="48">
         <v>2.5</v>
       </c>
       <c r="F38" s="48">
-        <v>5.0</v>
+        <v>3.5</v>
       </c>
       <c r="G38" s="48">
+        <v>4.5</v>
+      </c>
+      <c r="H38" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="I38" s="48">
         <v>3.5</v>
-      </c>
-      <c r="H38" s="48">
-        <v>1.5</v>
-      </c>
-      <c r="I38" s="48">
-        <v>2.0</v>
       </c>
       <c r="J38" s="49" t="s">
         <v>102</v>
       </c>
       <c r="K38" s="50">
-        <v>26.5</v>
+        <v>27.0</v>
       </c>
       <c r="L38" s="51">
-        <v>26.25</v>
+        <v>26.75</v>
       </c>
       <c r="M38" s="52">
         <f t="shared" si="1"/>
-        <v>0.65625</v>
+        <v>0.66875</v>
       </c>
       <c r="N38" s="53" t="s">
-        <v>45</v>
+        <v>87</v>
       </c>
       <c r="P38" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K38,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -2946,41 +2948,41 @@
         <v>3.5</v>
       </c>
       <c r="C39" s="48">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="D39" s="48">
         <v>2.5</v>
       </c>
       <c r="E39" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="F39" s="48">
+        <v>4.5</v>
+      </c>
+      <c r="G39" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="H39" s="48">
         <v>3.5</v>
       </c>
-      <c r="F39" s="48">
-        <v>3.5</v>
-      </c>
-      <c r="G39" s="48">
-        <v>5.0</v>
-      </c>
-      <c r="H39" s="48">
-        <v>2.5</v>
-      </c>
       <c r="I39" s="48">
-        <v>1.5</v>
+        <v>4.0</v>
       </c>
       <c r="J39" s="49" t="s">
         <v>104</v>
       </c>
       <c r="K39" s="50">
-        <v>26.0</v>
+        <v>27.0</v>
       </c>
       <c r="L39" s="51">
-        <v>25.75</v>
+        <v>26.5</v>
       </c>
       <c r="M39" s="52">
         <f t="shared" si="1"/>
-        <v>0.64375</v>
+        <v>0.6625</v>
       </c>
       <c r="N39" s="53" t="s">
-        <v>87</v>
+        <v>63</v>
       </c>
       <c r="P39" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K39,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -2988,48 +2990,48 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="47" t="s">
+      <c r="A40" s="57" t="s">
         <v>105</v>
       </c>
       <c r="B40" s="48">
+        <v>4.5</v>
+      </c>
+      <c r="C40" s="48">
         <v>3.5</v>
       </c>
-      <c r="C40" s="48">
-        <v>3.0</v>
-      </c>
       <c r="D40" s="48">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="E40" s="48">
         <v>2.5</v>
       </c>
       <c r="F40" s="48">
-        <v>3.0</v>
+        <v>5.0</v>
       </c>
       <c r="G40" s="48">
-        <v>4.5</v>
+        <v>3.5</v>
       </c>
       <c r="H40" s="48">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="I40" s="48">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
       <c r="J40" s="49" t="s">
         <v>106</v>
       </c>
       <c r="K40" s="50">
-        <v>26.0</v>
+        <v>26.5</v>
       </c>
       <c r="L40" s="51">
-        <v>25.75</v>
+        <v>26.25</v>
       </c>
       <c r="M40" s="52">
         <f t="shared" si="1"/>
-        <v>0.64375</v>
+        <v>0.65625</v>
       </c>
       <c r="N40" s="53" t="s">
-        <v>87</v>
+        <v>45</v>
       </c>
       <c r="P40" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K40,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3041,90 +3043,93 @@
         <v>107</v>
       </c>
       <c r="B41" s="48">
+        <v>3.5</v>
+      </c>
+      <c r="C41" s="48">
         <v>4.0</v>
-      </c>
-      <c r="C41" s="48">
-        <v>2.5</v>
       </c>
       <c r="D41" s="48">
         <v>2.5</v>
       </c>
       <c r="E41" s="48">
+        <v>3.5</v>
+      </c>
+      <c r="F41" s="48">
+        <v>3.5</v>
+      </c>
+      <c r="G41" s="48">
+        <v>5.0</v>
+      </c>
+      <c r="H41" s="48">
         <v>2.5</v>
       </c>
-      <c r="F41" s="48">
-        <v>3.0</v>
-      </c>
-      <c r="G41" s="48">
-        <v>4.5</v>
-      </c>
-      <c r="H41" s="48">
-        <v>2.0</v>
-      </c>
       <c r="I41" s="48">
-        <v>4.0</v>
+        <v>1.5</v>
       </c>
       <c r="J41" s="49" t="s">
         <v>108</v>
       </c>
       <c r="K41" s="50">
-        <v>25.0</v>
+        <v>26.0</v>
       </c>
       <c r="L41" s="51">
-        <v>25.0</v>
+        <v>25.75</v>
       </c>
       <c r="M41" s="52">
         <f t="shared" si="1"/>
-        <v>0.625</v>
+        <v>0.64375</v>
       </c>
       <c r="N41" s="53" t="s">
         <v>87</v>
       </c>
-      <c r="P41" s="54"/>
+      <c r="P41" s="54" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K41,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="47" t="s">
         <v>109</v>
       </c>
       <c r="B42" s="48">
+        <v>3.5</v>
+      </c>
+      <c r="C42" s="48">
         <v>3.0</v>
       </c>
-      <c r="C42" s="48">
+      <c r="D42" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="E42" s="48">
         <v>2.5</v>
-      </c>
-      <c r="D42" s="48">
-        <v>5.0</v>
-      </c>
-      <c r="E42" s="48">
-        <v>2.0</v>
       </c>
       <c r="F42" s="48">
         <v>3.0</v>
       </c>
       <c r="G42" s="48">
-        <v>5.0</v>
+        <v>4.5</v>
       </c>
       <c r="H42" s="48">
-        <v>2.0</v>
+        <v>2.5</v>
       </c>
       <c r="I42" s="48">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="J42" s="49" t="s">
         <v>110</v>
       </c>
       <c r="K42" s="50">
-        <v>24.5</v>
+        <v>26.0</v>
       </c>
       <c r="L42" s="51">
-        <v>24.25</v>
+        <v>25.75</v>
       </c>
       <c r="M42" s="52">
         <f t="shared" si="1"/>
-        <v>0.60625</v>
+        <v>0.64375</v>
       </c>
       <c r="N42" s="53" t="s">
-        <v>111</v>
+        <v>87</v>
       </c>
       <c r="P42" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K42,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3133,96 +3138,93 @@
     </row>
     <row r="43">
       <c r="A43" s="47" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B43" s="48">
-        <v>3.5</v>
+        <v>4.0</v>
       </c>
       <c r="C43" s="48">
-        <v>4.0</v>
+        <v>2.5</v>
       </c>
       <c r="D43" s="48">
         <v>2.5</v>
       </c>
       <c r="E43" s="48">
-        <v>3.0</v>
+        <v>2.5</v>
       </c>
       <c r="F43" s="48">
         <v>3.0</v>
       </c>
       <c r="G43" s="48">
-        <v>5.0</v>
+        <v>4.5</v>
       </c>
       <c r="H43" s="48">
         <v>2.0</v>
       </c>
       <c r="I43" s="48">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="J43" s="49" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="K43" s="50">
-        <v>24.0</v>
+        <v>25.0</v>
       </c>
       <c r="L43" s="51">
-        <v>23.75</v>
+        <v>25.0</v>
       </c>
       <c r="M43" s="52">
         <f t="shared" si="1"/>
-        <v>0.59375</v>
+        <v>0.625</v>
       </c>
       <c r="N43" s="53" t="s">
         <v>87</v>
       </c>
-      <c r="P43" s="54" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K43,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
-        <v/>
-      </c>
+      <c r="P43" s="54"/>
     </row>
     <row r="44">
       <c r="A44" s="47" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B44" s="48">
-        <v>3.5</v>
+        <v>3.0</v>
       </c>
       <c r="C44" s="48">
         <v>2.5</v>
       </c>
       <c r="D44" s="48">
-        <v>2.0</v>
+        <v>5.0</v>
       </c>
       <c r="E44" s="48">
         <v>2.0</v>
       </c>
       <c r="F44" s="48">
-        <v>3.5</v>
+        <v>3.0</v>
       </c>
       <c r="G44" s="48">
-        <v>4.5</v>
+        <v>5.0</v>
       </c>
       <c r="H44" s="48">
         <v>2.0</v>
       </c>
       <c r="I44" s="48">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
       <c r="J44" s="49" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K44" s="50">
-        <v>24.0</v>
+        <v>24.5</v>
       </c>
       <c r="L44" s="51">
-        <v>23.75</v>
+        <v>24.25</v>
       </c>
       <c r="M44" s="52">
         <f t="shared" si="1"/>
-        <v>0.59375</v>
+        <v>0.60625</v>
       </c>
       <c r="N44" s="53" t="s">
-        <v>87</v>
+        <v>115</v>
       </c>
       <c r="P44" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K44,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3249,7 +3251,7 @@
         <v>3.0</v>
       </c>
       <c r="G45" s="48">
-        <v>4.5</v>
+        <v>5.0</v>
       </c>
       <c r="H45" s="48">
         <v>2.0</v>
@@ -3261,63 +3263,66 @@
         <v>117</v>
       </c>
       <c r="K45" s="50">
-        <v>23.5</v>
+        <v>24.0</v>
       </c>
       <c r="L45" s="51">
-        <v>23.25</v>
+        <v>23.75</v>
       </c>
       <c r="M45" s="52">
         <f t="shared" si="1"/>
-        <v>0.58125</v>
+        <v>0.59375</v>
       </c>
       <c r="N45" s="53" t="s">
         <v>87</v>
       </c>
-      <c r="P45" s="54"/>
+      <c r="P45" s="54" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K45,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="47" t="s">
         <v>118</v>
       </c>
       <c r="B46" s="48">
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
       <c r="C46" s="48">
-        <v>4.0</v>
+        <v>2.5</v>
       </c>
       <c r="D46" s="48">
-        <v>5.0</v>
+        <v>2.0</v>
       </c>
       <c r="E46" s="48">
         <v>2.0</v>
       </c>
       <c r="F46" s="48">
-        <v>0.0</v>
+        <v>3.5</v>
       </c>
       <c r="G46" s="48">
-        <v>5.0</v>
+        <v>4.5</v>
       </c>
       <c r="H46" s="48">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="I46" s="48">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="J46" s="49" t="s">
         <v>119</v>
       </c>
       <c r="K46" s="50">
-        <v>20.5</v>
+        <v>24.0</v>
       </c>
       <c r="L46" s="51">
-        <v>20.25</v>
+        <v>23.75</v>
       </c>
       <c r="M46" s="52">
         <f t="shared" si="1"/>
-        <v>0.50625</v>
+        <v>0.59375</v>
       </c>
       <c r="N46" s="53" t="s">
-        <v>111</v>
+        <v>87</v>
       </c>
       <c r="P46" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K46,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3325,97 +3330,94 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="57" t="s">
+      <c r="A47" s="47" t="s">
         <v>120</v>
       </c>
       <c r="B47" s="48">
-        <v>0.0</v>
+        <v>3.5</v>
       </c>
       <c r="C47" s="48">
-        <v>1.5</v>
+        <v>4.0</v>
       </c>
       <c r="D47" s="48">
-        <v>3.0</v>
+        <v>2.5</v>
       </c>
       <c r="E47" s="48">
         <v>3.0</v>
       </c>
       <c r="F47" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="G47" s="48">
         <v>4.5</v>
-      </c>
-      <c r="G47" s="48">
-        <v>2.0</v>
       </c>
       <c r="H47" s="48">
         <v>2.0</v>
       </c>
       <c r="I47" s="48">
-        <v>3.5</v>
+        <v>1.0</v>
       </c>
       <c r="J47" s="49" t="s">
         <v>121</v>
       </c>
       <c r="K47" s="50">
-        <v>19.5</v>
+        <v>23.5</v>
       </c>
       <c r="L47" s="51">
-        <v>19.25</v>
+        <v>23.25</v>
       </c>
       <c r="M47" s="52">
         <f t="shared" si="1"/>
-        <v>0.48125</v>
+        <v>0.58125</v>
       </c>
       <c r="N47" s="53" t="s">
-        <v>111</v>
-      </c>
-      <c r="P47" s="54" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K47,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
-        <v/>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="P47" s="54"/>
     </row>
     <row r="48">
-      <c r="A48" s="57" t="s">
+      <c r="A48" s="47" t="s">
         <v>122</v>
       </c>
       <c r="B48" s="48">
-        <v>3.0</v>
+        <v>1.5</v>
       </c>
       <c r="C48" s="48">
-        <v>2.5</v>
+        <v>4.0</v>
       </c>
       <c r="D48" s="48">
-        <v>2.5</v>
+        <v>5.0</v>
       </c>
       <c r="E48" s="48">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="F48" s="48">
-        <v>0.5</v>
+        <v>0.0</v>
       </c>
       <c r="G48" s="48">
+        <v>5.0</v>
+      </c>
+      <c r="H48" s="48">
+        <v>1.0</v>
+      </c>
+      <c r="I48" s="48">
         <v>2.0</v>
-      </c>
-      <c r="H48" s="48">
-        <v>2.0</v>
-      </c>
-      <c r="I48" s="48">
-        <v>4.0</v>
       </c>
       <c r="J48" s="49" t="s">
         <v>123</v>
       </c>
       <c r="K48" s="50">
-        <v>19.5</v>
+        <v>20.5</v>
       </c>
       <c r="L48" s="51">
-        <v>19.0</v>
+        <v>20.25</v>
       </c>
       <c r="M48" s="52">
         <f t="shared" si="1"/>
-        <v>0.475</v>
+        <v>0.50625</v>
       </c>
       <c r="N48" s="53" t="s">
-        <v>87</v>
+        <v>115</v>
       </c>
       <c r="P48" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K48,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3427,44 +3429,44 @@
         <v>124</v>
       </c>
       <c r="B49" s="48">
-        <v>0.5</v>
+        <v>0.0</v>
       </c>
       <c r="C49" s="48">
+        <v>1.5</v>
+      </c>
+      <c r="D49" s="48">
         <v>3.0</v>
       </c>
-      <c r="D49" s="48">
-        <v>3.5</v>
-      </c>
       <c r="E49" s="48">
-        <v>2.5</v>
+        <v>3.0</v>
       </c>
       <c r="F49" s="48">
-        <v>0.0</v>
+        <v>4.5</v>
       </c>
       <c r="G49" s="48">
         <v>2.0</v>
       </c>
       <c r="H49" s="48">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="I49" s="48">
-        <v>3.0</v>
+        <v>3.5</v>
       </c>
       <c r="J49" s="49" t="s">
         <v>125</v>
       </c>
       <c r="K49" s="50">
-        <v>15.5</v>
+        <v>19.5</v>
       </c>
       <c r="L49" s="51">
-        <v>15.25</v>
+        <v>19.25</v>
       </c>
       <c r="M49" s="52">
         <f t="shared" si="1"/>
-        <v>0.38125</v>
+        <v>0.48125</v>
       </c>
       <c r="N49" s="53" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="P49" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K49,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3476,41 +3478,41 @@
         <v>126</v>
       </c>
       <c r="B50" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="C50" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="D50" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="E50" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="F50" s="48">
         <v>0.5</v>
       </c>
-      <c r="C50" s="48">
-        <v>0.0</v>
-      </c>
-      <c r="D50" s="48">
-        <v>0.5</v>
-      </c>
-      <c r="E50" s="48">
-        <v>0.5</v>
-      </c>
-      <c r="F50" s="48">
-        <v>0.0</v>
-      </c>
       <c r="G50" s="48">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="H50" s="48">
-        <v>0.5</v>
+        <v>2.0</v>
       </c>
       <c r="I50" s="48">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="J50" s="49" t="s">
         <v>127</v>
       </c>
       <c r="K50" s="50">
-        <v>6.5</v>
+        <v>19.5</v>
       </c>
       <c r="L50" s="51">
-        <v>6.25</v>
+        <v>19.0</v>
       </c>
       <c r="M50" s="52">
         <f t="shared" si="1"/>
-        <v>0.15625</v>
+        <v>0.475</v>
       </c>
       <c r="N50" s="53" t="s">
         <v>87</v>
@@ -3521,48 +3523,48 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="58" t="s">
+      <c r="A51" s="57" t="s">
         <v>128</v>
       </c>
-      <c r="B51" s="59">
+      <c r="B51" s="48">
+        <v>0.5</v>
+      </c>
+      <c r="C51" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="D51" s="48">
+        <v>3.5</v>
+      </c>
+      <c r="E51" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="F51" s="48">
+        <v>0.0</v>
+      </c>
+      <c r="G51" s="48">
+        <v>2.0</v>
+      </c>
+      <c r="H51" s="48">
         <v>1.0</v>
       </c>
-      <c r="C51" s="59">
-        <v>0.0</v>
-      </c>
-      <c r="D51" s="59">
-        <v>0.5</v>
-      </c>
-      <c r="E51" s="59">
-        <v>0.5</v>
-      </c>
-      <c r="F51" s="59">
-        <v>0.0</v>
-      </c>
-      <c r="G51" s="59">
-        <v>0.0</v>
-      </c>
-      <c r="H51" s="59">
-        <v>0.5</v>
-      </c>
-      <c r="I51" s="59">
-        <v>0.5</v>
-      </c>
-      <c r="J51" s="60" t="s">
+      <c r="I51" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="J51" s="49" t="s">
         <v>129</v>
       </c>
-      <c r="K51" s="61">
-        <v>3.5</v>
-      </c>
-      <c r="L51" s="62">
-        <v>3.25</v>
+      <c r="K51" s="50">
+        <v>15.5</v>
+      </c>
+      <c r="L51" s="51">
+        <v>15.25</v>
       </c>
       <c r="M51" s="52">
         <f t="shared" si="1"/>
-        <v>0.08125</v>
+        <v>0.38125</v>
       </c>
       <c r="N51" s="53" t="s">
-        <v>87</v>
+        <v>115</v>
       </c>
       <c r="P51" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K51,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3570,20 +3572,102 @@
       </c>
     </row>
     <row r="52">
-      <c r="J52" s="63"/>
-      <c r="K52" s="64"/>
-      <c r="L52" s="65"/>
-      <c r="M52" s="66"/>
-      <c r="N52" s="67"/>
-      <c r="P52" s="68"/>
+      <c r="A52" s="57" t="s">
+        <v>130</v>
+      </c>
+      <c r="B52" s="48">
+        <v>0.5</v>
+      </c>
+      <c r="C52" s="48">
+        <v>0.0</v>
+      </c>
+      <c r="D52" s="48">
+        <v>0.5</v>
+      </c>
+      <c r="E52" s="48">
+        <v>0.5</v>
+      </c>
+      <c r="F52" s="48">
+        <v>0.0</v>
+      </c>
+      <c r="G52" s="48">
+        <v>1.0</v>
+      </c>
+      <c r="H52" s="48">
+        <v>0.5</v>
+      </c>
+      <c r="I52" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="J52" s="49" t="s">
+        <v>131</v>
+      </c>
+      <c r="K52" s="50">
+        <v>6.5</v>
+      </c>
+      <c r="L52" s="51">
+        <v>6.25</v>
+      </c>
+      <c r="M52" s="52">
+        <f t="shared" si="1"/>
+        <v>0.15625</v>
+      </c>
+      <c r="N52" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="P52" s="54" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K52,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
-      <c r="J53" s="63"/>
-      <c r="K53" s="64"/>
-      <c r="L53" s="65"/>
-      <c r="M53" s="66"/>
-      <c r="N53" s="67"/>
-      <c r="P53" s="68"/>
+      <c r="A53" s="58" t="s">
+        <v>132</v>
+      </c>
+      <c r="B53" s="59">
+        <v>1.0</v>
+      </c>
+      <c r="C53" s="59">
+        <v>0.0</v>
+      </c>
+      <c r="D53" s="59">
+        <v>0.5</v>
+      </c>
+      <c r="E53" s="59">
+        <v>0.5</v>
+      </c>
+      <c r="F53" s="59">
+        <v>0.0</v>
+      </c>
+      <c r="G53" s="59">
+        <v>0.0</v>
+      </c>
+      <c r="H53" s="59">
+        <v>0.5</v>
+      </c>
+      <c r="I53" s="59">
+        <v>0.5</v>
+      </c>
+      <c r="J53" s="60" t="s">
+        <v>133</v>
+      </c>
+      <c r="K53" s="61">
+        <v>3.5</v>
+      </c>
+      <c r="L53" s="62">
+        <v>3.25</v>
+      </c>
+      <c r="M53" s="52">
+        <f t="shared" si="1"/>
+        <v>0.08125</v>
+      </c>
+      <c r="N53" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="P53" s="54" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K53,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="J54" s="63"/>
@@ -11201,19 +11285,35 @@
       <c r="N1005" s="67"/>
       <c r="P1005" s="68"/>
     </row>
+    <row r="1006">
+      <c r="J1006" s="63"/>
+      <c r="K1006" s="64"/>
+      <c r="L1006" s="65"/>
+      <c r="M1006" s="66"/>
+      <c r="N1006" s="67"/>
+      <c r="P1006" s="68"/>
+    </row>
+    <row r="1007">
+      <c r="J1007" s="63"/>
+      <c r="K1007" s="64"/>
+      <c r="L1007" s="65"/>
+      <c r="M1007" s="66"/>
+      <c r="N1007" s="67"/>
+      <c r="P1007" s="68"/>
+    </row>
   </sheetData>
-  <autoFilter ref="$A$7:$P$51">
-    <sortState ref="A7:P51">
-      <sortCondition descending="1" ref="L7:L51"/>
-      <sortCondition descending="1" ref="P7:P51"/>
-      <sortCondition descending="1" ref="I7:I51"/>
-      <sortCondition descending="1" ref="F7:F51"/>
-      <sortCondition descending="1" ref="H7:H51"/>
-      <sortCondition descending="1" ref="G7:G51"/>
-      <sortCondition descending="1" ref="E7:E51"/>
-      <sortCondition descending="1" ref="D7:D51"/>
-      <sortCondition descending="1" ref="C7:C51"/>
-      <sortCondition descending="1" ref="B7:B51"/>
+  <autoFilter ref="$A$7:$P$53">
+    <sortState ref="A7:P53">
+      <sortCondition descending="1" ref="L7:L53"/>
+      <sortCondition descending="1" ref="P7:P53"/>
+      <sortCondition descending="1" ref="I7:I53"/>
+      <sortCondition descending="1" ref="F7:F53"/>
+      <sortCondition descending="1" ref="H7:H53"/>
+      <sortCondition descending="1" ref="G7:G53"/>
+      <sortCondition descending="1" ref="E7:E53"/>
+      <sortCondition descending="1" ref="D7:D53"/>
+      <sortCondition descending="1" ref="C7:C53"/>
+      <sortCondition descending="1" ref="B7:B53"/>
     </sortState>
   </autoFilter>
   <mergeCells count="3">
@@ -11221,7 +11321,7 @@
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="G4:H4"/>
   </mergeCells>
-  <conditionalFormatting sqref="B8:I51">
+  <conditionalFormatting sqref="B8:I53">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -11234,7 +11334,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="N8:N51">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="N8:N53">
       <formula1>"C,S,P,A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add round v4.9 files (WarShare formalization, re-audit)
</commit_message>
<xml_diff>
--- a/assets/ledger.xlsx
+++ b/assets/ledger.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="136">
   <si>
     <t>Civ-likeness Rating System</t>
   </si>
@@ -101,7 +101,8 @@
     <t>Q-field (quarter-precision total, derived from unrounded P6b/P7 components)</t>
   </si>
   <si>
-    <t>War-Share. Levels: Core / Substantial / Peripheral / Absent.</t>
+    <t>War-Share: position on the builder↔wargame axis of the ancestral duality — the wargame tradition's share of the design (military systems + conquest teleology; adversarialness alone is not war-share). Orthogonal to the pillar metrics
+Levels: Pure (~100%) Core (~75%) / Substantial (~50%) / Peripheral (~25%) / Absent (~0%) or N/A.</t>
   </si>
   <si>
     <t>Game</t>
@@ -152,7 +153,7 @@
     <t>30.0/10.0</t>
   </si>
   <si>
-    <t>S</t>
+    <t>50 %</t>
   </si>
   <si>
     <t>Civ6 (2016, GS)</t>
@@ -206,7 +207,7 @@
     <t>29.0/8.5</t>
   </si>
   <si>
-    <t>P</t>
+    <t>25 %</t>
   </si>
   <si>
     <t>Civ1 (1991)</t>
@@ -278,7 +279,7 @@
     <t>25.0/7.5</t>
   </si>
   <si>
-    <t>C</t>
+    <t>75 %</t>
   </si>
   <si>
     <t>Anno 1800 (2019–2022)</t>
@@ -320,6 +321,9 @@
     <t>24.0/5.5</t>
   </si>
   <si>
+    <t>100 %</t>
+  </si>
+  <si>
     <t>Total War: Warhammer III (2022, IE + 9.0)</t>
   </si>
   <si>
@@ -362,7 +366,7 @@
     <t>19.5/5.0</t>
   </si>
   <si>
-    <t>A</t>
+    <t>0 %</t>
   </si>
   <si>
     <t>StarCraft II (melee, vs-AI)</t>
@@ -399,6 +403,9 @@
   </si>
   <si>
     <t>17.0/2.5</t>
+  </si>
+  <si>
+    <t>N/A</t>
   </si>
   <si>
     <t>The Sims 4 (live)</t>
@@ -426,7 +433,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="42">
+  <fonts count="41">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -566,12 +573,6 @@
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="8.0"/>
-      <color theme="1"/>
-      <name val="Arial"/>
     </font>
     <font>
       <b/>
@@ -799,120 +800,120 @@
     <xf borderId="0" fillId="0" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="2" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="2" fontId="14" numFmtId="2" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    <xf borderId="0" fillId="0" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="25" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="25" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="24" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="16" numFmtId="2" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="26" numFmtId="10" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="25" numFmtId="10" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="28" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="29" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="1" fillId="2" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="27" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="28" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="1" fillId="2" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="2" fontId="29" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="30" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="31" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="24" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="25" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="2" fontId="31" numFmtId="2" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="32" numFmtId="2" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="2" fontId="32" numFmtId="10" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="33" numFmtId="10" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="2" fontId="33" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="34" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="35" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="34" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="35" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="3" fontId="34" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="35" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="34" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="36" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="5" fontId="35" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="37" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="4" fontId="36" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="35" numFmtId="10" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="4" fontId="34" numFmtId="10" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="38" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="37" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="39" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="38" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="40" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="39" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="35" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="4" fontId="34" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="40" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="39" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="40" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="39" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="35" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="3" fontId="34" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="35" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="34" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="5" fontId="36" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="5" fontId="35" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="37" numFmtId="2" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="4" fontId="36" numFmtId="2" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="28" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="27" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="17" numFmtId="2" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="41" numFmtId="10" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="40" numFmtId="10" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="29" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="39" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="0" fontId="38" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -1134,7 +1135,8 @@
     <col customWidth="1" min="2" max="9" width="20.13"/>
     <col customWidth="1" min="10" max="10" width="28.88"/>
     <col customWidth="1" min="11" max="12" width="11.38"/>
-    <col customWidth="1" min="13" max="14" width="8.88"/>
+    <col customWidth="1" min="13" max="13" width="8.88"/>
+    <col customWidth="1" min="14" max="14" width="17.63"/>
     <col customWidth="1" min="15" max="16" width="6.38"/>
   </cols>
   <sheetData>
@@ -1317,15 +1319,15 @@
       <c r="I5" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="J5" s="17" t="s">
+      <c r="J5" s="29" t="s">
         <v>26</v>
       </c>
       <c r="K5" s="25"/>
-      <c r="L5" s="29" t="s">
+      <c r="L5" s="30" t="s">
         <v>27</v>
       </c>
       <c r="M5" s="27"/>
-      <c r="N5" s="30" t="s">
+      <c r="N5" s="29" t="s">
         <v>28</v>
       </c>
       <c r="O5" s="28"/>
@@ -2502,7 +2504,7 @@
         <v>0.85625</v>
       </c>
       <c r="N29" s="53" t="s">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="P29" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K29,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -2648,7 +2650,9 @@
         <f t="shared" si="1"/>
         <v>0.79375</v>
       </c>
-      <c r="N32" s="53"/>
+      <c r="N32" s="53" t="s">
+        <v>87</v>
+      </c>
       <c r="P32" s="54"/>
     </row>
     <row r="33">
@@ -2888,12 +2892,14 @@
         <f t="shared" si="1"/>
         <v>0.73125</v>
       </c>
-      <c r="N37" s="53"/>
+      <c r="N37" s="53" t="s">
+        <v>101</v>
+      </c>
       <c r="P37" s="54"/>
     </row>
     <row r="38">
       <c r="A38" s="47" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B38" s="48">
         <v>4.5</v>
@@ -2920,7 +2926,7 @@
         <v>3.5</v>
       </c>
       <c r="J38" s="49" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K38" s="50">
         <v>27.0</v>
@@ -2942,7 +2948,7 @@
     </row>
     <row r="39">
       <c r="A39" s="47" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B39" s="48">
         <v>3.5</v>
@@ -2969,7 +2975,7 @@
         <v>4.0</v>
       </c>
       <c r="J39" s="49" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K39" s="50">
         <v>27.0</v>
@@ -2982,7 +2988,7 @@
         <v>0.6625</v>
       </c>
       <c r="N39" s="53" t="s">
-        <v>63</v>
+        <v>45</v>
       </c>
       <c r="P39" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K39,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -2991,7 +2997,7 @@
     </row>
     <row r="40">
       <c r="A40" s="57" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B40" s="48">
         <v>4.5</v>
@@ -3018,7 +3024,7 @@
         <v>2.0</v>
       </c>
       <c r="J40" s="49" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K40" s="50">
         <v>26.5</v>
@@ -3040,7 +3046,7 @@
     </row>
     <row r="41">
       <c r="A41" s="47" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B41" s="48">
         <v>3.5</v>
@@ -3067,7 +3073,7 @@
         <v>1.5</v>
       </c>
       <c r="J41" s="49" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K41" s="50">
         <v>26.0</v>
@@ -3089,7 +3095,7 @@
     </row>
     <row r="42">
       <c r="A42" s="47" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B42" s="48">
         <v>3.5</v>
@@ -3116,7 +3122,7 @@
         <v>4.0</v>
       </c>
       <c r="J42" s="49" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K42" s="50">
         <v>26.0</v>
@@ -3129,7 +3135,7 @@
         <v>0.64375</v>
       </c>
       <c r="N42" s="53" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="P42" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K42,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3138,7 +3144,7 @@
     </row>
     <row r="43">
       <c r="A43" s="47" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B43" s="48">
         <v>4.0</v>
@@ -3165,7 +3171,7 @@
         <v>4.0</v>
       </c>
       <c r="J43" s="49" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K43" s="50">
         <v>25.0</v>
@@ -3178,13 +3184,13 @@
         <v>0.625</v>
       </c>
       <c r="N43" s="53" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="P43" s="54"/>
     </row>
     <row r="44">
       <c r="A44" s="47" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B44" s="48">
         <v>3.0</v>
@@ -3211,7 +3217,7 @@
         <v>2.0</v>
       </c>
       <c r="J44" s="49" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K44" s="50">
         <v>24.5</v>
@@ -3224,7 +3230,7 @@
         <v>0.60625</v>
       </c>
       <c r="N44" s="53" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P44" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K44,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3233,7 +3239,7 @@
     </row>
     <row r="45">
       <c r="A45" s="47" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B45" s="48">
         <v>3.5</v>
@@ -3260,7 +3266,7 @@
         <v>1.0</v>
       </c>
       <c r="J45" s="49" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K45" s="50">
         <v>24.0</v>
@@ -3273,7 +3279,7 @@
         <v>0.59375</v>
       </c>
       <c r="N45" s="53" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="P45" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K45,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3282,7 +3288,7 @@
     </row>
     <row r="46">
       <c r="A46" s="47" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B46" s="48">
         <v>3.5</v>
@@ -3309,7 +3315,7 @@
         <v>4.0</v>
       </c>
       <c r="J46" s="49" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K46" s="50">
         <v>24.0</v>
@@ -3331,7 +3337,7 @@
     </row>
     <row r="47">
       <c r="A47" s="47" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B47" s="48">
         <v>3.5</v>
@@ -3358,7 +3364,7 @@
         <v>1.0</v>
       </c>
       <c r="J47" s="49" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="K47" s="50">
         <v>23.5</v>
@@ -3371,13 +3377,13 @@
         <v>0.58125</v>
       </c>
       <c r="N47" s="53" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="P47" s="54"/>
     </row>
     <row r="48">
       <c r="A48" s="47" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B48" s="48">
         <v>1.5</v>
@@ -3404,7 +3410,7 @@
         <v>2.0</v>
       </c>
       <c r="J48" s="49" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="K48" s="50">
         <v>20.5</v>
@@ -3417,7 +3423,7 @@
         <v>0.50625</v>
       </c>
       <c r="N48" s="53" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P48" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K48,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3426,7 +3432,7 @@
     </row>
     <row r="49">
       <c r="A49" s="57" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B49" s="48">
         <v>0.0</v>
@@ -3453,7 +3459,7 @@
         <v>3.5</v>
       </c>
       <c r="J49" s="49" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K49" s="50">
         <v>19.5</v>
@@ -3466,7 +3472,7 @@
         <v>0.48125</v>
       </c>
       <c r="N49" s="53" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P49" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K49,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3475,7 +3481,7 @@
     </row>
     <row r="50">
       <c r="A50" s="57" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B50" s="48">
         <v>3.0</v>
@@ -3502,7 +3508,7 @@
         <v>4.0</v>
       </c>
       <c r="J50" s="49" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="K50" s="50">
         <v>19.5</v>
@@ -3515,7 +3521,7 @@
         <v>0.475</v>
       </c>
       <c r="N50" s="53" t="s">
-        <v>87</v>
+        <v>129</v>
       </c>
       <c r="P50" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K50,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3524,7 +3530,7 @@
     </row>
     <row r="51">
       <c r="A51" s="57" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B51" s="48">
         <v>0.5</v>
@@ -3551,7 +3557,7 @@
         <v>3.0</v>
       </c>
       <c r="J51" s="49" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="K51" s="50">
         <v>15.5</v>
@@ -3564,7 +3570,7 @@
         <v>0.38125</v>
       </c>
       <c r="N51" s="53" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P51" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K51,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3573,7 +3579,7 @@
     </row>
     <row r="52">
       <c r="A52" s="57" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B52" s="48">
         <v>0.5</v>
@@ -3600,7 +3606,7 @@
         <v>3.0</v>
       </c>
       <c r="J52" s="49" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="K52" s="50">
         <v>6.5</v>
@@ -3613,7 +3619,7 @@
         <v>0.15625</v>
       </c>
       <c r="N52" s="53" t="s">
-        <v>87</v>
+        <v>129</v>
       </c>
       <c r="P52" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K52,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3622,7 +3628,7 @@
     </row>
     <row r="53">
       <c r="A53" s="58" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B53" s="59">
         <v>1.0</v>
@@ -3649,7 +3655,7 @@
         <v>0.5</v>
       </c>
       <c r="J53" s="60" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="K53" s="61">
         <v>3.5</v>
@@ -3662,7 +3668,7 @@
         <v>0.08125</v>
       </c>
       <c r="N53" s="53" t="s">
-        <v>87</v>
+        <v>129</v>
       </c>
       <c r="P53" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K53,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -11335,7 +11341,7 @@
   </conditionalFormatting>
   <dataValidations>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="N8:N53">
-      <formula1>"C,S,P,A"</formula1>
+      <formula1>"100 %,75 %,50 %,25 %,0 %,N/A"</formula1>
     </dataValidation>
   </dataValidations>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Plot the round v4.10 (Conquest of Eo + Fantasy General)
</commit_message>
<xml_diff>
--- a/assets/ledger.xlsx
+++ b/assets/ledger.xlsx
@@ -6,14 +6,14 @@
     <sheet state="visible" name="ledger" sheetId="1" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">ledger!$A$7:$P$53</definedName>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">ledger!$A$7:$P$55</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="140">
   <si>
     <t>Civ-likeness Rating System</t>
   </si>
@@ -324,6 +324,12 @@
     <t>100 %</t>
   </si>
   <si>
+    <t>SpellForce: Conquest of Eo (2023–25, +3 DLC)</t>
+  </si>
+  <si>
+    <t>22.0/5.5</t>
+  </si>
+  <si>
     <t>Total War: Warhammer III (2022, IE + 9.0)</t>
   </si>
   <si>
@@ -406,6 +412,12 @@
   </si>
   <si>
     <t>N/A</t>
+  </si>
+  <si>
+    <t>Fantasy General (1996, +Island Challenge)</t>
+  </si>
+  <si>
+    <t>12.5/3.5</t>
   </si>
   <si>
     <t>The Sims 4 (live)</t>
@@ -1480,7 +1492,7 @@
         <v>40.0</v>
       </c>
       <c r="M8" s="52">
-        <f t="shared" ref="M8:M53" si="1">L8/40</f>
+        <f t="shared" ref="M8:M55" si="1">L8/40</f>
         <v>1</v>
       </c>
       <c r="N8" s="53" t="s">
@@ -2902,56 +2914,53 @@
         <v>102</v>
       </c>
       <c r="B38" s="48">
-        <v>4.5</v>
+        <v>4.0</v>
       </c>
       <c r="C38" s="48">
         <v>3.0</v>
       </c>
       <c r="D38" s="48">
+        <v>4.0</v>
+      </c>
+      <c r="E38" s="48">
+        <v>3.5</v>
+      </c>
+      <c r="F38" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="G38" s="48">
+        <v>3.5</v>
+      </c>
+      <c r="H38" s="48">
         <v>2.5</v>
       </c>
-      <c r="E38" s="48">
-        <v>2.5</v>
-      </c>
-      <c r="F38" s="48">
-        <v>3.5</v>
-      </c>
-      <c r="G38" s="48">
-        <v>4.5</v>
-      </c>
-      <c r="H38" s="48">
-        <v>3.0</v>
-      </c>
       <c r="I38" s="48">
-        <v>3.5</v>
+        <v>4.0</v>
       </c>
       <c r="J38" s="49" t="s">
         <v>103</v>
       </c>
       <c r="K38" s="50">
-        <v>27.0</v>
+        <v>27.5</v>
       </c>
       <c r="L38" s="51">
-        <v>26.75</v>
+        <v>27.5</v>
       </c>
       <c r="M38" s="52">
         <f t="shared" si="1"/>
-        <v>0.66875</v>
+        <v>0.6875</v>
       </c>
       <c r="N38" s="53" t="s">
         <v>87</v>
       </c>
-      <c r="P38" s="54" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K38,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
-        <v/>
-      </c>
+      <c r="P38" s="54"/>
     </row>
     <row r="39">
       <c r="A39" s="47" t="s">
         <v>104</v>
       </c>
       <c r="B39" s="48">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="C39" s="48">
         <v>3.0</v>
@@ -2960,19 +2969,19 @@
         <v>2.5</v>
       </c>
       <c r="E39" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="F39" s="48">
+        <v>3.5</v>
+      </c>
+      <c r="G39" s="48">
+        <v>4.5</v>
+      </c>
+      <c r="H39" s="48">
         <v>3.0</v>
       </c>
-      <c r="F39" s="48">
-        <v>4.5</v>
-      </c>
-      <c r="G39" s="48">
-        <v>3.0</v>
-      </c>
-      <c r="H39" s="48">
+      <c r="I39" s="48">
         <v>3.5</v>
-      </c>
-      <c r="I39" s="48">
-        <v>4.0</v>
       </c>
       <c r="J39" s="49" t="s">
         <v>105</v>
@@ -2981,14 +2990,14 @@
         <v>27.0</v>
       </c>
       <c r="L39" s="51">
-        <v>26.5</v>
+        <v>26.75</v>
       </c>
       <c r="M39" s="52">
         <f t="shared" si="1"/>
-        <v>0.6625</v>
+        <v>0.66875</v>
       </c>
       <c r="N39" s="53" t="s">
-        <v>45</v>
+        <v>87</v>
       </c>
       <c r="P39" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K39,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -2996,45 +3005,45 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="57" t="s">
+      <c r="A40" s="47" t="s">
         <v>106</v>
       </c>
       <c r="B40" s="48">
+        <v>3.5</v>
+      </c>
+      <c r="C40" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="D40" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="E40" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="F40" s="48">
         <v>4.5</v>
       </c>
-      <c r="C40" s="48">
+      <c r="G40" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="H40" s="48">
         <v>3.5</v>
       </c>
-      <c r="D40" s="48">
+      <c r="I40" s="48">
         <v>4.0</v>
-      </c>
-      <c r="E40" s="48">
-        <v>2.5</v>
-      </c>
-      <c r="F40" s="48">
-        <v>5.0</v>
-      </c>
-      <c r="G40" s="48">
-        <v>3.5</v>
-      </c>
-      <c r="H40" s="48">
-        <v>1.5</v>
-      </c>
-      <c r="I40" s="48">
-        <v>2.0</v>
       </c>
       <c r="J40" s="49" t="s">
         <v>107</v>
       </c>
       <c r="K40" s="50">
+        <v>27.0</v>
+      </c>
+      <c r="L40" s="51">
         <v>26.5</v>
-      </c>
-      <c r="L40" s="51">
-        <v>26.25</v>
       </c>
       <c r="M40" s="52">
         <f t="shared" si="1"/>
-        <v>0.65625</v>
+        <v>0.6625</v>
       </c>
       <c r="N40" s="53" t="s">
         <v>45</v>
@@ -3045,48 +3054,48 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="47" t="s">
+      <c r="A41" s="57" t="s">
         <v>108</v>
       </c>
       <c r="B41" s="48">
+        <v>4.5</v>
+      </c>
+      <c r="C41" s="48">
         <v>3.5</v>
       </c>
-      <c r="C41" s="48">
+      <c r="D41" s="48">
         <v>4.0</v>
       </c>
-      <c r="D41" s="48">
+      <c r="E41" s="48">
         <v>2.5</v>
       </c>
-      <c r="E41" s="48">
+      <c r="F41" s="48">
+        <v>5.0</v>
+      </c>
+      <c r="G41" s="48">
         <v>3.5</v>
       </c>
-      <c r="F41" s="48">
-        <v>3.5</v>
-      </c>
-      <c r="G41" s="48">
-        <v>5.0</v>
-      </c>
       <c r="H41" s="48">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="I41" s="48">
-        <v>1.5</v>
+        <v>2.0</v>
       </c>
       <c r="J41" s="49" t="s">
         <v>109</v>
       </c>
       <c r="K41" s="50">
-        <v>26.0</v>
+        <v>26.5</v>
       </c>
       <c r="L41" s="51">
-        <v>25.75</v>
+        <v>26.25</v>
       </c>
       <c r="M41" s="52">
         <f t="shared" si="1"/>
-        <v>0.64375</v>
+        <v>0.65625</v>
       </c>
       <c r="N41" s="53" t="s">
-        <v>87</v>
+        <v>45</v>
       </c>
       <c r="P41" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K41,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3101,25 +3110,25 @@
         <v>3.5</v>
       </c>
       <c r="C42" s="48">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="D42" s="48">
-        <v>3.0</v>
+        <v>2.5</v>
       </c>
       <c r="E42" s="48">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="F42" s="48">
-        <v>3.0</v>
+        <v>3.5</v>
       </c>
       <c r="G42" s="48">
-        <v>4.5</v>
+        <v>5.0</v>
       </c>
       <c r="H42" s="48">
         <v>2.5</v>
       </c>
       <c r="I42" s="48">
-        <v>4.0</v>
+        <v>1.5</v>
       </c>
       <c r="J42" s="49" t="s">
         <v>111</v>
@@ -3135,7 +3144,7 @@
         <v>0.64375</v>
       </c>
       <c r="N42" s="53" t="s">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="P42" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K42,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3147,13 +3156,13 @@
         <v>112</v>
       </c>
       <c r="B43" s="48">
-        <v>4.0</v>
+        <v>3.5</v>
       </c>
       <c r="C43" s="48">
-        <v>2.5</v>
+        <v>3.0</v>
       </c>
       <c r="D43" s="48">
-        <v>2.5</v>
+        <v>3.0</v>
       </c>
       <c r="E43" s="48">
         <v>2.5</v>
@@ -3165,7 +3174,7 @@
         <v>4.5</v>
       </c>
       <c r="H43" s="48">
-        <v>2.0</v>
+        <v>2.5</v>
       </c>
       <c r="I43" s="48">
         <v>4.0</v>
@@ -3174,84 +3183,84 @@
         <v>113</v>
       </c>
       <c r="K43" s="50">
-        <v>25.0</v>
+        <v>26.0</v>
       </c>
       <c r="L43" s="51">
-        <v>25.0</v>
+        <v>25.75</v>
       </c>
       <c r="M43" s="52">
         <f t="shared" si="1"/>
-        <v>0.625</v>
+        <v>0.64375</v>
       </c>
       <c r="N43" s="53" t="s">
         <v>101</v>
       </c>
-      <c r="P43" s="54"/>
+      <c r="P43" s="54" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K43,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="47" t="s">
         <v>114</v>
       </c>
       <c r="B44" s="48">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="C44" s="48">
         <v>2.5</v>
       </c>
       <c r="D44" s="48">
-        <v>5.0</v>
+        <v>2.5</v>
       </c>
       <c r="E44" s="48">
-        <v>2.0</v>
+        <v>2.5</v>
       </c>
       <c r="F44" s="48">
         <v>3.0</v>
       </c>
       <c r="G44" s="48">
-        <v>5.0</v>
+        <v>4.5</v>
       </c>
       <c r="H44" s="48">
         <v>2.0</v>
       </c>
       <c r="I44" s="48">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="J44" s="49" t="s">
         <v>115</v>
       </c>
       <c r="K44" s="50">
-        <v>24.5</v>
+        <v>25.0</v>
       </c>
       <c r="L44" s="51">
-        <v>24.25</v>
+        <v>25.0</v>
       </c>
       <c r="M44" s="52">
         <f t="shared" si="1"/>
-        <v>0.60625</v>
+        <v>0.625</v>
       </c>
       <c r="N44" s="53" t="s">
-        <v>116</v>
-      </c>
-      <c r="P44" s="54" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K44,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
-        <v/>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="P44" s="54"/>
     </row>
     <row r="45">
       <c r="A45" s="47" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B45" s="48">
-        <v>3.5</v>
+        <v>3.0</v>
       </c>
       <c r="C45" s="48">
-        <v>4.0</v>
+        <v>2.5</v>
       </c>
       <c r="D45" s="48">
-        <v>2.5</v>
+        <v>5.0</v>
       </c>
       <c r="E45" s="48">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="F45" s="48">
         <v>3.0</v>
@@ -3263,23 +3272,23 @@
         <v>2.0</v>
       </c>
       <c r="I45" s="48">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="J45" s="49" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="K45" s="50">
-        <v>24.0</v>
+        <v>24.5</v>
       </c>
       <c r="L45" s="51">
-        <v>23.75</v>
+        <v>24.25</v>
       </c>
       <c r="M45" s="52">
         <f t="shared" si="1"/>
-        <v>0.59375</v>
+        <v>0.60625</v>
       </c>
       <c r="N45" s="53" t="s">
-        <v>101</v>
+        <v>118</v>
       </c>
       <c r="P45" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K45,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3294,25 +3303,25 @@
         <v>3.5</v>
       </c>
       <c r="C46" s="48">
+        <v>4.0</v>
+      </c>
+      <c r="D46" s="48">
         <v>2.5</v>
       </c>
-      <c r="D46" s="48">
-        <v>2.0</v>
-      </c>
       <c r="E46" s="48">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="F46" s="48">
-        <v>3.5</v>
+        <v>3.0</v>
       </c>
       <c r="G46" s="48">
-        <v>4.5</v>
+        <v>5.0</v>
       </c>
       <c r="H46" s="48">
         <v>2.0</v>
       </c>
       <c r="I46" s="48">
-        <v>4.0</v>
+        <v>1.0</v>
       </c>
       <c r="J46" s="49" t="s">
         <v>120</v>
@@ -3328,7 +3337,7 @@
         <v>0.59375</v>
       </c>
       <c r="N46" s="53" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="P46" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K46,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3343,16 +3352,16 @@
         <v>3.5</v>
       </c>
       <c r="C47" s="48">
-        <v>4.0</v>
+        <v>2.5</v>
       </c>
       <c r="D47" s="48">
-        <v>2.5</v>
+        <v>2.0</v>
       </c>
       <c r="E47" s="48">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="F47" s="48">
-        <v>3.0</v>
+        <v>3.5</v>
       </c>
       <c r="G47" s="48">
         <v>4.5</v>
@@ -3361,118 +3370,118 @@
         <v>2.0</v>
       </c>
       <c r="I47" s="48">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="J47" s="49" t="s">
         <v>122</v>
       </c>
       <c r="K47" s="50">
-        <v>23.5</v>
+        <v>24.0</v>
       </c>
       <c r="L47" s="51">
-        <v>23.25</v>
+        <v>23.75</v>
       </c>
       <c r="M47" s="52">
         <f t="shared" si="1"/>
-        <v>0.58125</v>
+        <v>0.59375</v>
       </c>
       <c r="N47" s="53" t="s">
-        <v>101</v>
-      </c>
-      <c r="P47" s="54"/>
+        <v>87</v>
+      </c>
+      <c r="P47" s="54" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K47,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="47" t="s">
         <v>123</v>
       </c>
       <c r="B48" s="48">
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
       <c r="C48" s="48">
         <v>4.0</v>
       </c>
       <c r="D48" s="48">
-        <v>5.0</v>
+        <v>2.5</v>
       </c>
       <c r="E48" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="F48" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="G48" s="48">
+        <v>4.5</v>
+      </c>
+      <c r="H48" s="48">
         <v>2.0</v>
       </c>
-      <c r="F48" s="48">
-        <v>0.0</v>
-      </c>
-      <c r="G48" s="48">
-        <v>5.0</v>
-      </c>
-      <c r="H48" s="48">
+      <c r="I48" s="48">
         <v>1.0</v>
-      </c>
-      <c r="I48" s="48">
-        <v>2.0</v>
       </c>
       <c r="J48" s="49" t="s">
         <v>124</v>
       </c>
       <c r="K48" s="50">
-        <v>20.5</v>
+        <v>23.5</v>
       </c>
       <c r="L48" s="51">
-        <v>20.25</v>
+        <v>23.25</v>
       </c>
       <c r="M48" s="52">
         <f t="shared" si="1"/>
-        <v>0.50625</v>
+        <v>0.58125</v>
       </c>
       <c r="N48" s="53" t="s">
-        <v>116</v>
-      </c>
-      <c r="P48" s="54" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K48,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
-        <v/>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="P48" s="54"/>
     </row>
     <row r="49">
-      <c r="A49" s="57" t="s">
+      <c r="A49" s="47" t="s">
         <v>125</v>
       </c>
       <c r="B49" s="48">
+        <v>1.5</v>
+      </c>
+      <c r="C49" s="48">
+        <v>4.0</v>
+      </c>
+      <c r="D49" s="48">
+        <v>5.0</v>
+      </c>
+      <c r="E49" s="48">
+        <v>2.0</v>
+      </c>
+      <c r="F49" s="48">
         <v>0.0</v>
       </c>
-      <c r="C49" s="48">
-        <v>1.5</v>
-      </c>
-      <c r="D49" s="48">
-        <v>3.0</v>
-      </c>
-      <c r="E49" s="48">
-        <v>3.0</v>
-      </c>
-      <c r="F49" s="48">
-        <v>4.5</v>
-      </c>
       <c r="G49" s="48">
+        <v>5.0</v>
+      </c>
+      <c r="H49" s="48">
+        <v>1.0</v>
+      </c>
+      <c r="I49" s="48">
         <v>2.0</v>
-      </c>
-      <c r="H49" s="48">
-        <v>2.0</v>
-      </c>
-      <c r="I49" s="48">
-        <v>3.5</v>
       </c>
       <c r="J49" s="49" t="s">
         <v>126</v>
       </c>
       <c r="K49" s="50">
-        <v>19.5</v>
+        <v>20.5</v>
       </c>
       <c r="L49" s="51">
-        <v>19.25</v>
+        <v>20.25</v>
       </c>
       <c r="M49" s="52">
         <f t="shared" si="1"/>
-        <v>0.48125</v>
+        <v>0.50625</v>
       </c>
       <c r="N49" s="53" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="P49" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K49,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3484,19 +3493,19 @@
         <v>127</v>
       </c>
       <c r="B50" s="48">
+        <v>0.0</v>
+      </c>
+      <c r="C50" s="48">
+        <v>1.5</v>
+      </c>
+      <c r="D50" s="48">
         <v>3.0</v>
-      </c>
-      <c r="C50" s="48">
-        <v>2.5</v>
-      </c>
-      <c r="D50" s="48">
-        <v>2.5</v>
       </c>
       <c r="E50" s="48">
         <v>3.0</v>
       </c>
       <c r="F50" s="48">
-        <v>0.5</v>
+        <v>4.5</v>
       </c>
       <c r="G50" s="48">
         <v>2.0</v>
@@ -3505,7 +3514,7 @@
         <v>2.0</v>
       </c>
       <c r="I50" s="48">
-        <v>4.0</v>
+        <v>3.5</v>
       </c>
       <c r="J50" s="49" t="s">
         <v>128</v>
@@ -3514,14 +3523,14 @@
         <v>19.5</v>
       </c>
       <c r="L50" s="51">
-        <v>19.0</v>
+        <v>19.25</v>
       </c>
       <c r="M50" s="52">
         <f t="shared" si="1"/>
-        <v>0.475</v>
+        <v>0.48125</v>
       </c>
       <c r="N50" s="53" t="s">
-        <v>129</v>
+        <v>118</v>
       </c>
       <c r="P50" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K50,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3530,47 +3539,47 @@
     </row>
     <row r="51">
       <c r="A51" s="57" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B51" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="C51" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="D51" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="E51" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="F51" s="48">
         <v>0.5</v>
-      </c>
-      <c r="C51" s="48">
-        <v>3.0</v>
-      </c>
-      <c r="D51" s="48">
-        <v>3.5</v>
-      </c>
-      <c r="E51" s="48">
-        <v>2.5</v>
-      </c>
-      <c r="F51" s="48">
-        <v>0.0</v>
       </c>
       <c r="G51" s="48">
         <v>2.0</v>
       </c>
       <c r="H51" s="48">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="I51" s="48">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="J51" s="49" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="K51" s="50">
-        <v>15.5</v>
+        <v>19.5</v>
       </c>
       <c r="L51" s="51">
-        <v>15.25</v>
+        <v>19.0</v>
       </c>
       <c r="M51" s="52">
         <f t="shared" si="1"/>
-        <v>0.38125</v>
+        <v>0.475</v>
       </c>
       <c r="N51" s="53" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="P51" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K51,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3582,93 +3591,90 @@
         <v>132</v>
       </c>
       <c r="B52" s="48">
+        <v>1.5</v>
+      </c>
+      <c r="C52" s="48">
         <v>0.5</v>
       </c>
-      <c r="C52" s="48">
-        <v>0.0</v>
-      </c>
       <c r="D52" s="48">
-        <v>0.5</v>
+        <v>2.0</v>
       </c>
       <c r="E52" s="48">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="F52" s="48">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="G52" s="48">
-        <v>1.0</v>
+        <v>3.5</v>
       </c>
       <c r="H52" s="48">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="I52" s="48">
-        <v>3.0</v>
+        <v>3.5</v>
       </c>
       <c r="J52" s="49" t="s">
         <v>133</v>
       </c>
       <c r="K52" s="50">
-        <v>6.5</v>
+        <v>16.0</v>
       </c>
       <c r="L52" s="51">
-        <v>6.25</v>
+        <v>15.75</v>
       </c>
       <c r="M52" s="52">
         <f t="shared" si="1"/>
-        <v>0.15625</v>
+        <v>0.39375</v>
       </c>
       <c r="N52" s="53" t="s">
-        <v>129</v>
-      </c>
-      <c r="P52" s="54" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K52,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
-        <v/>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="P52" s="54"/>
     </row>
     <row r="53">
-      <c r="A53" s="58" t="s">
+      <c r="A53" s="57" t="s">
         <v>134</v>
       </c>
-      <c r="B53" s="59">
+      <c r="B53" s="48">
+        <v>0.5</v>
+      </c>
+      <c r="C53" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="D53" s="48">
+        <v>3.5</v>
+      </c>
+      <c r="E53" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="F53" s="48">
+        <v>0.0</v>
+      </c>
+      <c r="G53" s="48">
+        <v>2.0</v>
+      </c>
+      <c r="H53" s="48">
         <v>1.0</v>
       </c>
-      <c r="C53" s="59">
-        <v>0.0</v>
-      </c>
-      <c r="D53" s="59">
-        <v>0.5</v>
-      </c>
-      <c r="E53" s="59">
-        <v>0.5</v>
-      </c>
-      <c r="F53" s="59">
-        <v>0.0</v>
-      </c>
-      <c r="G53" s="59">
-        <v>0.0</v>
-      </c>
-      <c r="H53" s="59">
-        <v>0.5</v>
-      </c>
-      <c r="I53" s="59">
-        <v>0.5</v>
-      </c>
-      <c r="J53" s="60" t="s">
+      <c r="I53" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="J53" s="49" t="s">
         <v>135</v>
       </c>
-      <c r="K53" s="61">
-        <v>3.5</v>
-      </c>
-      <c r="L53" s="62">
-        <v>3.25</v>
+      <c r="K53" s="50">
+        <v>15.5</v>
+      </c>
+      <c r="L53" s="51">
+        <v>15.25</v>
       </c>
       <c r="M53" s="52">
         <f t="shared" si="1"/>
-        <v>0.08125</v>
+        <v>0.38125</v>
       </c>
       <c r="N53" s="53" t="s">
-        <v>129</v>
+        <v>118</v>
       </c>
       <c r="P53" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K53,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3676,20 +3682,102 @@
       </c>
     </row>
     <row r="54">
-      <c r="J54" s="63"/>
-      <c r="K54" s="64"/>
-      <c r="L54" s="65"/>
-      <c r="M54" s="66"/>
-      <c r="N54" s="67"/>
-      <c r="P54" s="68"/>
+      <c r="A54" s="57" t="s">
+        <v>136</v>
+      </c>
+      <c r="B54" s="48">
+        <v>0.5</v>
+      </c>
+      <c r="C54" s="48">
+        <v>0.0</v>
+      </c>
+      <c r="D54" s="48">
+        <v>0.5</v>
+      </c>
+      <c r="E54" s="48">
+        <v>0.5</v>
+      </c>
+      <c r="F54" s="48">
+        <v>0.0</v>
+      </c>
+      <c r="G54" s="48">
+        <v>1.0</v>
+      </c>
+      <c r="H54" s="48">
+        <v>0.5</v>
+      </c>
+      <c r="I54" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="J54" s="49" t="s">
+        <v>137</v>
+      </c>
+      <c r="K54" s="50">
+        <v>6.5</v>
+      </c>
+      <c r="L54" s="51">
+        <v>6.25</v>
+      </c>
+      <c r="M54" s="52">
+        <f t="shared" si="1"/>
+        <v>0.15625</v>
+      </c>
+      <c r="N54" s="53" t="s">
+        <v>131</v>
+      </c>
+      <c r="P54" s="54" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K54,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
-      <c r="J55" s="63"/>
-      <c r="K55" s="64"/>
-      <c r="L55" s="65"/>
-      <c r="M55" s="66"/>
-      <c r="N55" s="67"/>
-      <c r="P55" s="68"/>
+      <c r="A55" s="58" t="s">
+        <v>138</v>
+      </c>
+      <c r="B55" s="59">
+        <v>1.0</v>
+      </c>
+      <c r="C55" s="59">
+        <v>0.0</v>
+      </c>
+      <c r="D55" s="59">
+        <v>0.5</v>
+      </c>
+      <c r="E55" s="59">
+        <v>0.5</v>
+      </c>
+      <c r="F55" s="59">
+        <v>0.0</v>
+      </c>
+      <c r="G55" s="59">
+        <v>0.0</v>
+      </c>
+      <c r="H55" s="59">
+        <v>0.5</v>
+      </c>
+      <c r="I55" s="59">
+        <v>0.5</v>
+      </c>
+      <c r="J55" s="60" t="s">
+        <v>139</v>
+      </c>
+      <c r="K55" s="61">
+        <v>3.5</v>
+      </c>
+      <c r="L55" s="62">
+        <v>3.25</v>
+      </c>
+      <c r="M55" s="52">
+        <f t="shared" si="1"/>
+        <v>0.08125</v>
+      </c>
+      <c r="N55" s="53" t="s">
+        <v>131</v>
+      </c>
+      <c r="P55" s="54" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K55,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="J56" s="63"/>
@@ -11307,19 +11395,35 @@
       <c r="N1007" s="67"/>
       <c r="P1007" s="68"/>
     </row>
+    <row r="1008">
+      <c r="J1008" s="63"/>
+      <c r="K1008" s="64"/>
+      <c r="L1008" s="65"/>
+      <c r="M1008" s="66"/>
+      <c r="N1008" s="67"/>
+      <c r="P1008" s="68"/>
+    </row>
+    <row r="1009">
+      <c r="J1009" s="63"/>
+      <c r="K1009" s="64"/>
+      <c r="L1009" s="65"/>
+      <c r="M1009" s="66"/>
+      <c r="N1009" s="67"/>
+      <c r="P1009" s="68"/>
+    </row>
   </sheetData>
-  <autoFilter ref="$A$7:$P$53">
-    <sortState ref="A7:P53">
-      <sortCondition descending="1" ref="L7:L53"/>
-      <sortCondition descending="1" ref="P7:P53"/>
-      <sortCondition descending="1" ref="I7:I53"/>
-      <sortCondition descending="1" ref="F7:F53"/>
-      <sortCondition descending="1" ref="H7:H53"/>
-      <sortCondition descending="1" ref="G7:G53"/>
-      <sortCondition descending="1" ref="E7:E53"/>
-      <sortCondition descending="1" ref="D7:D53"/>
-      <sortCondition descending="1" ref="C7:C53"/>
-      <sortCondition descending="1" ref="B7:B53"/>
+  <autoFilter ref="$A$7:$P$55">
+    <sortState ref="A7:P55">
+      <sortCondition descending="1" ref="L7:L55"/>
+      <sortCondition descending="1" ref="P7:P55"/>
+      <sortCondition descending="1" ref="I7:I55"/>
+      <sortCondition descending="1" ref="F7:F55"/>
+      <sortCondition descending="1" ref="H7:H55"/>
+      <sortCondition descending="1" ref="G7:G55"/>
+      <sortCondition descending="1" ref="E7:E55"/>
+      <sortCondition descending="1" ref="D7:D55"/>
+      <sortCondition descending="1" ref="C7:C55"/>
+      <sortCondition descending="1" ref="B7:B55"/>
     </sortState>
   </autoFilter>
   <mergeCells count="3">
@@ -11327,7 +11431,7 @@
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="G4:H4"/>
   </mergeCells>
-  <conditionalFormatting sqref="B8:I53">
+  <conditionalFormatting sqref="B8:I55">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -11340,7 +11444,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="N8:N53">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="N8:N55">
       <formula1>"100 %,75 %,50 %,25 %,0 %,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Plot the round v4.12 (Populous+B&W)
</commit_message>
<xml_diff>
--- a/assets/ledger.xlsx
+++ b/assets/ledger.xlsx
@@ -6,14 +6,14 @@
     <sheet state="visible" name="ledger" sheetId="1" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">ledger!$A$7:$P$55</definedName>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">ledger!$A$7:$P$57</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="143">
   <si>
     <t>Civ-likeness Rating System</t>
   </si>
@@ -399,6 +399,9 @@
     <t>19.5/1.0</t>
   </si>
   <si>
+    <t>N/A</t>
+  </si>
+  <si>
     <t>Football Manager 26 (final)</t>
   </si>
   <si>
@@ -411,9 +414,6 @@
     <t>17.0/2.5</t>
   </si>
   <si>
-    <t>N/A</t>
-  </si>
-  <si>
     <t>Fantasy General (1996, +Island Challenge)</t>
   </si>
   <si>
@@ -424,6 +424,15 @@
   </si>
   <si>
     <t>14.5/1.0</t>
+  </si>
+  <si>
+    <t>Populous (1989, +The Promised Lands)</t>
+  </si>
+  <si>
+    <t>11.0/4.0</t>
+  </si>
+  <si>
+    <t>Black &amp; White (2001, +Creature Isle)</t>
   </si>
   <si>
     <t>Into the Breach (2018, AE)</t>
@@ -1511,7 +1520,7 @@
         <v>40.0</v>
       </c>
       <c r="M8" s="52">
-        <f t="shared" ref="M8:M55" si="1">L8/40</f>
+        <f t="shared" ref="M8:M57" si="1">L8/40</f>
         <v>1</v>
       </c>
       <c r="N8" s="53" t="s">
@@ -3500,7 +3509,7 @@
         <v>0.50625</v>
       </c>
       <c r="N49" s="53" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="P49" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K49,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3509,7 +3518,7 @@
     </row>
     <row r="50">
       <c r="A50" s="60" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B50" s="48">
         <v>0.0</v>
@@ -3536,7 +3545,7 @@
         <v>3.5</v>
       </c>
       <c r="J50" s="49" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K50" s="50">
         <v>19.5</v>
@@ -3558,7 +3567,7 @@
     </row>
     <row r="51">
       <c r="A51" s="60" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B51" s="48">
         <v>3.0</v>
@@ -3585,7 +3594,7 @@
         <v>4.0</v>
       </c>
       <c r="J51" s="49" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K51" s="50">
         <v>19.5</v>
@@ -3598,7 +3607,7 @@
         <v>0.475</v>
       </c>
       <c r="N51" s="53" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="P51" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K51,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3693,7 +3702,7 @@
         <v>0.38125</v>
       </c>
       <c r="N53" s="53" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="P53" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K53,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3705,114 +3714,190 @@
         <v>136</v>
       </c>
       <c r="B54" s="48">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="C54" s="48">
-        <v>0.0</v>
+        <v>2.5</v>
       </c>
       <c r="D54" s="48">
-        <v>0.5</v>
+        <v>2.0</v>
       </c>
       <c r="E54" s="48">
         <v>0.5</v>
       </c>
       <c r="F54" s="48">
-        <v>0.0</v>
+        <v>3.0</v>
       </c>
       <c r="G54" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="H54" s="48">
         <v>1.0</v>
       </c>
-      <c r="H54" s="48">
-        <v>0.5</v>
-      </c>
       <c r="I54" s="48">
-        <v>3.0</v>
+        <v>1.5</v>
       </c>
       <c r="J54" s="49" t="s">
         <v>137</v>
       </c>
       <c r="K54" s="50">
-        <v>6.5</v>
+        <v>15.0</v>
       </c>
       <c r="L54" s="51">
-        <v>6.25</v>
+        <v>15.0</v>
       </c>
       <c r="M54" s="52">
         <f t="shared" si="1"/>
-        <v>0.15625</v>
+        <v>0.375</v>
       </c>
       <c r="N54" s="53" t="s">
-        <v>131</v>
-      </c>
-      <c r="P54" s="54" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K54,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
-        <v/>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="P54" s="54"/>
     </row>
     <row r="55">
-      <c r="A55" s="61" t="s">
+      <c r="A55" s="47" t="s">
         <v>138</v>
       </c>
-      <c r="B55" s="62">
-        <v>1.0</v>
-      </c>
-      <c r="C55" s="62">
-        <v>0.0</v>
-      </c>
-      <c r="D55" s="62">
+      <c r="B55" s="48">
+        <v>1.5</v>
+      </c>
+      <c r="C55" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="D55" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="E55" s="48">
         <v>0.5</v>
       </c>
-      <c r="E55" s="62">
-        <v>0.5</v>
-      </c>
-      <c r="F55" s="62">
-        <v>0.0</v>
-      </c>
-      <c r="G55" s="62">
-        <v>0.0</v>
-      </c>
-      <c r="H55" s="62">
-        <v>0.5</v>
-      </c>
-      <c r="I55" s="62">
-        <v>0.5</v>
-      </c>
-      <c r="J55" s="63" t="s">
-        <v>139</v>
-      </c>
-      <c r="K55" s="64">
-        <v>3.5</v>
-      </c>
-      <c r="L55" s="65">
-        <v>3.25</v>
+      <c r="F55" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="G55" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="H55" s="48">
+        <v>1.5</v>
+      </c>
+      <c r="I55" s="48">
+        <v>1.5</v>
+      </c>
+      <c r="J55" s="49" t="s">
+        <v>137</v>
+      </c>
+      <c r="K55" s="50">
+        <v>15.0</v>
+      </c>
+      <c r="L55" s="51">
+        <v>15.0</v>
       </c>
       <c r="M55" s="52">
         <f t="shared" si="1"/>
+        <v>0.375</v>
+      </c>
+      <c r="N55" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="P55" s="54"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="60" t="s">
+        <v>139</v>
+      </c>
+      <c r="B56" s="48">
+        <v>0.5</v>
+      </c>
+      <c r="C56" s="48">
+        <v>0.0</v>
+      </c>
+      <c r="D56" s="48">
+        <v>0.5</v>
+      </c>
+      <c r="E56" s="48">
+        <v>0.5</v>
+      </c>
+      <c r="F56" s="48">
+        <v>0.0</v>
+      </c>
+      <c r="G56" s="48">
+        <v>1.0</v>
+      </c>
+      <c r="H56" s="48">
+        <v>0.5</v>
+      </c>
+      <c r="I56" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="J56" s="49" t="s">
+        <v>140</v>
+      </c>
+      <c r="K56" s="50">
+        <v>6.5</v>
+      </c>
+      <c r="L56" s="51">
+        <v>6.25</v>
+      </c>
+      <c r="M56" s="52">
+        <f t="shared" si="1"/>
+        <v>0.15625</v>
+      </c>
+      <c r="N56" s="53" t="s">
+        <v>127</v>
+      </c>
+      <c r="P56" s="54" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K56,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="61" t="s">
+        <v>141</v>
+      </c>
+      <c r="B57" s="62">
+        <v>1.0</v>
+      </c>
+      <c r="C57" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="D57" s="62">
+        <v>0.5</v>
+      </c>
+      <c r="E57" s="62">
+        <v>0.5</v>
+      </c>
+      <c r="F57" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="G57" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="H57" s="62">
+        <v>0.5</v>
+      </c>
+      <c r="I57" s="62">
+        <v>0.5</v>
+      </c>
+      <c r="J57" s="63" t="s">
+        <v>142</v>
+      </c>
+      <c r="K57" s="64">
+        <v>3.5</v>
+      </c>
+      <c r="L57" s="65">
+        <v>3.25</v>
+      </c>
+      <c r="M57" s="52">
+        <f t="shared" si="1"/>
         <v>0.08125</v>
       </c>
-      <c r="N55" s="53" t="s">
-        <v>131</v>
-      </c>
-      <c r="P55" s="54" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K55,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
+      <c r="N57" s="53" t="s">
+        <v>127</v>
+      </c>
+      <c r="P57" s="54" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K57,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="56">
-      <c r="J56" s="66"/>
-      <c r="K56" s="67"/>
-      <c r="L56" s="68"/>
-      <c r="M56" s="69"/>
-      <c r="N56" s="70"/>
-      <c r="P56" s="71"/>
-    </row>
-    <row r="57">
-      <c r="J57" s="66"/>
-      <c r="K57" s="67"/>
-      <c r="L57" s="68"/>
-      <c r="M57" s="69"/>
-      <c r="N57" s="70"/>
-      <c r="P57" s="71"/>
     </row>
     <row r="58">
       <c r="J58" s="66"/>
@@ -11430,19 +11515,35 @@
       <c r="N1009" s="70"/>
       <c r="P1009" s="71"/>
     </row>
+    <row r="1010">
+      <c r="J1010" s="66"/>
+      <c r="K1010" s="67"/>
+      <c r="L1010" s="68"/>
+      <c r="M1010" s="69"/>
+      <c r="N1010" s="70"/>
+      <c r="P1010" s="71"/>
+    </row>
+    <row r="1011">
+      <c r="J1011" s="66"/>
+      <c r="K1011" s="67"/>
+      <c r="L1011" s="68"/>
+      <c r="M1011" s="69"/>
+      <c r="N1011" s="70"/>
+      <c r="P1011" s="71"/>
+    </row>
   </sheetData>
-  <autoFilter ref="$A$7:$P$55">
-    <sortState ref="A7:P55">
-      <sortCondition descending="1" ref="L7:L55"/>
-      <sortCondition descending="1" ref="P7:P55"/>
-      <sortCondition descending="1" ref="I7:I55"/>
-      <sortCondition descending="1" ref="F7:F55"/>
-      <sortCondition descending="1" ref="H7:H55"/>
-      <sortCondition descending="1" ref="G7:G55"/>
-      <sortCondition descending="1" ref="E7:E55"/>
-      <sortCondition descending="1" ref="D7:D55"/>
-      <sortCondition descending="1" ref="C7:C55"/>
-      <sortCondition descending="1" ref="B7:B55"/>
+  <autoFilter ref="$A$7:$P$57">
+    <sortState ref="A7:P57">
+      <sortCondition descending="1" ref="L7:L57"/>
+      <sortCondition descending="1" ref="P7:P57"/>
+      <sortCondition descending="1" ref="I7:I57"/>
+      <sortCondition descending="1" ref="F7:F57"/>
+      <sortCondition descending="1" ref="H7:H57"/>
+      <sortCondition descending="1" ref="G7:G57"/>
+      <sortCondition descending="1" ref="E7:E57"/>
+      <sortCondition descending="1" ref="D7:D57"/>
+      <sortCondition descending="1" ref="C7:C57"/>
+      <sortCondition descending="1" ref="B7:B57"/>
     </sortState>
   </autoFilter>
   <mergeCells count="3">
@@ -11450,7 +11551,7 @@
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="G4:H4"/>
   </mergeCells>
-  <conditionalFormatting sqref="B8:I55">
+  <conditionalFormatting sqref="B8:I57">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -11463,7 +11564,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="N8:N55">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="N8:N57">
       <formula1>"100 %,75 %,50 %,25 %,0 %,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Plot the round v4.13 (Songs of Conquest + Eador: Genesis)
</commit_message>
<xml_diff>
--- a/assets/ledger.xlsx
+++ b/assets/ledger.xlsx
@@ -6,14 +6,14 @@
     <sheet state="visible" name="ledger" sheetId="1" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">ledger!$A$7:$P$57</definedName>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">ledger!$A$7:$P$59</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="145">
   <si>
     <t>Civ-likeness Rating System</t>
   </si>
@@ -360,6 +360,9 @@
     <t>20.5/5.5</t>
   </si>
   <si>
+    <t>Songs of Conquest (2022–current, v1.4 + faction DLC)</t>
+  </si>
+  <si>
     <t>Conquest of Elysium 5 (2021–current)</t>
   </si>
   <si>
@@ -385,6 +388,9 @@
   </si>
   <si>
     <t>18.5/5.5</t>
+  </si>
+  <si>
+    <t>Eador: Genesis (2009–13, final)</t>
   </si>
   <si>
     <t>Warcraft III: TFT (2003, melee vs-AI)</t>
@@ -932,10 +938,10 @@
     <xf borderId="0" fillId="4" fontId="34" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="5" fontId="35" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="5" fontId="40" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="36" numFmtId="2" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="4" fontId="41" numFmtId="2" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -1171,7 +1177,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="39.13"/>
+    <col customWidth="1" min="1" max="1" width="41.25"/>
     <col customWidth="1" min="2" max="9" width="20.13"/>
     <col customWidth="1" min="10" max="10" width="28.88"/>
     <col customWidth="1" min="11" max="12" width="11.38"/>
@@ -1520,7 +1526,7 @@
         <v>40.0</v>
       </c>
       <c r="M8" s="52">
-        <f t="shared" ref="M8:M57" si="1">L8/40</f>
+        <f t="shared" ref="M8:M59" si="1">L8/40</f>
         <v>1</v>
       </c>
       <c r="N8" s="53" t="s">
@@ -3229,17 +3235,17 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="47" t="s">
+      <c r="A44" s="60" t="s">
         <v>114</v>
       </c>
       <c r="B44" s="48">
-        <v>4.0</v>
+        <v>3.5</v>
       </c>
       <c r="C44" s="48">
-        <v>2.5</v>
+        <v>3.0</v>
       </c>
       <c r="D44" s="48">
-        <v>2.5</v>
+        <v>3.0</v>
       </c>
       <c r="E44" s="48">
         <v>2.5</v>
@@ -3251,23 +3257,23 @@
         <v>4.5</v>
       </c>
       <c r="H44" s="48">
-        <v>2.0</v>
+        <v>2.5</v>
       </c>
       <c r="I44" s="48">
         <v>4.0</v>
       </c>
       <c r="J44" s="49" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="K44" s="50">
-        <v>25.0</v>
+        <v>26.0</v>
       </c>
       <c r="L44" s="51">
-        <v>25.0</v>
+        <v>25.5</v>
       </c>
       <c r="M44" s="52">
         <f t="shared" si="1"/>
-        <v>0.625</v>
+        <v>0.6375</v>
       </c>
       <c r="N44" s="53" t="s">
         <v>101</v>
@@ -3276,68 +3282,65 @@
     </row>
     <row r="45">
       <c r="A45" s="47" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B45" s="48">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="C45" s="48">
         <v>2.5</v>
       </c>
       <c r="D45" s="48">
-        <v>5.0</v>
+        <v>2.5</v>
       </c>
       <c r="E45" s="48">
-        <v>2.0</v>
+        <v>2.5</v>
       </c>
       <c r="F45" s="48">
         <v>3.0</v>
       </c>
       <c r="G45" s="48">
-        <v>5.0</v>
+        <v>4.5</v>
       </c>
       <c r="H45" s="48">
         <v>2.0</v>
       </c>
       <c r="I45" s="48">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="J45" s="49" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="K45" s="50">
-        <v>24.5</v>
+        <v>25.0</v>
       </c>
       <c r="L45" s="51">
-        <v>24.25</v>
+        <v>25.0</v>
       </c>
       <c r="M45" s="52">
         <f t="shared" si="1"/>
-        <v>0.60625</v>
+        <v>0.625</v>
       </c>
       <c r="N45" s="53" t="s">
-        <v>118</v>
-      </c>
-      <c r="P45" s="54" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K45,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
-        <v/>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="P45" s="54"/>
     </row>
     <row r="46">
       <c r="A46" s="47" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B46" s="48">
-        <v>3.5</v>
+        <v>3.0</v>
       </c>
       <c r="C46" s="48">
-        <v>4.0</v>
+        <v>2.5</v>
       </c>
       <c r="D46" s="48">
-        <v>2.5</v>
+        <v>5.0</v>
       </c>
       <c r="E46" s="48">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="F46" s="48">
         <v>3.0</v>
@@ -3349,23 +3352,23 @@
         <v>2.0</v>
       </c>
       <c r="I46" s="48">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="J46" s="49" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="K46" s="50">
-        <v>24.0</v>
+        <v>24.5</v>
       </c>
       <c r="L46" s="51">
-        <v>23.75</v>
+        <v>24.25</v>
       </c>
       <c r="M46" s="52">
         <f t="shared" si="1"/>
-        <v>0.59375</v>
+        <v>0.60625</v>
       </c>
       <c r="N46" s="53" t="s">
-        <v>101</v>
+        <v>119</v>
       </c>
       <c r="P46" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K46,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3374,34 +3377,34 @@
     </row>
     <row r="47">
       <c r="A47" s="47" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B47" s="48">
         <v>3.5</v>
       </c>
       <c r="C47" s="48">
+        <v>4.0</v>
+      </c>
+      <c r="D47" s="48">
         <v>2.5</v>
       </c>
-      <c r="D47" s="48">
-        <v>2.0</v>
-      </c>
       <c r="E47" s="48">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="F47" s="48">
-        <v>3.5</v>
+        <v>3.0</v>
       </c>
       <c r="G47" s="48">
-        <v>4.5</v>
+        <v>5.0</v>
       </c>
       <c r="H47" s="48">
         <v>2.0</v>
       </c>
       <c r="I47" s="48">
-        <v>4.0</v>
+        <v>1.0</v>
       </c>
       <c r="J47" s="49" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="K47" s="50">
         <v>24.0</v>
@@ -3414,7 +3417,7 @@
         <v>0.59375</v>
       </c>
       <c r="N47" s="53" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="P47" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K47,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3423,22 +3426,22 @@
     </row>
     <row r="48">
       <c r="A48" s="47" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B48" s="48">
         <v>3.5</v>
       </c>
       <c r="C48" s="48">
-        <v>4.0</v>
+        <v>2.5</v>
       </c>
       <c r="D48" s="48">
-        <v>2.5</v>
+        <v>2.0</v>
       </c>
       <c r="E48" s="48">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="F48" s="48">
-        <v>3.0</v>
+        <v>3.5</v>
       </c>
       <c r="G48" s="48">
         <v>4.5</v>
@@ -3447,167 +3450,164 @@
         <v>2.0</v>
       </c>
       <c r="I48" s="48">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="J48" s="49" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K48" s="50">
-        <v>23.5</v>
+        <v>24.0</v>
       </c>
       <c r="L48" s="51">
-        <v>23.25</v>
+        <v>23.75</v>
       </c>
       <c r="M48" s="52">
         <f t="shared" si="1"/>
-        <v>0.58125</v>
+        <v>0.59375</v>
       </c>
       <c r="N48" s="53" t="s">
-        <v>101</v>
-      </c>
-      <c r="P48" s="54"/>
+        <v>87</v>
+      </c>
+      <c r="P48" s="54" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K48,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="47" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B49" s="48">
-        <v>1.5</v>
+        <v>3.0</v>
       </c>
       <c r="C49" s="48">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
       <c r="D49" s="48">
-        <v>5.0</v>
+        <v>2.5</v>
       </c>
       <c r="E49" s="48">
         <v>2.0</v>
       </c>
       <c r="F49" s="48">
-        <v>0.0</v>
+        <v>3.5</v>
       </c>
       <c r="G49" s="48">
-        <v>5.0</v>
+        <v>4.0</v>
       </c>
       <c r="H49" s="48">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="I49" s="48">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="J49" s="49" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="K49" s="50">
-        <v>20.5</v>
-      </c>
-      <c r="L49" s="51">
-        <v>20.25</v>
+        <v>24.0</v>
+      </c>
+      <c r="L49" s="56">
+        <v>23.75</v>
       </c>
       <c r="M49" s="52">
         <f t="shared" si="1"/>
-        <v>0.50625</v>
+        <v>0.59375</v>
       </c>
       <c r="N49" s="53" t="s">
-        <v>127</v>
-      </c>
-      <c r="P49" s="54" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K49,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
-        <v/>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="P49" s="54"/>
     </row>
     <row r="50">
-      <c r="A50" s="60" t="s">
-        <v>128</v>
+      <c r="A50" s="47" t="s">
+        <v>125</v>
       </c>
       <c r="B50" s="48">
-        <v>0.0</v>
+        <v>3.5</v>
       </c>
       <c r="C50" s="48">
-        <v>1.5</v>
+        <v>4.0</v>
       </c>
       <c r="D50" s="48">
-        <v>3.0</v>
+        <v>2.5</v>
       </c>
       <c r="E50" s="48">
         <v>3.0</v>
       </c>
       <c r="F50" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="G50" s="48">
         <v>4.5</v>
-      </c>
-      <c r="G50" s="48">
-        <v>2.0</v>
       </c>
       <c r="H50" s="48">
         <v>2.0</v>
       </c>
       <c r="I50" s="48">
-        <v>3.5</v>
+        <v>1.0</v>
       </c>
       <c r="J50" s="49" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="K50" s="50">
-        <v>19.5</v>
+        <v>23.5</v>
       </c>
       <c r="L50" s="51">
-        <v>19.25</v>
+        <v>23.25</v>
       </c>
       <c r="M50" s="52">
         <f t="shared" si="1"/>
-        <v>0.48125</v>
+        <v>0.58125</v>
       </c>
       <c r="N50" s="53" t="s">
-        <v>118</v>
-      </c>
-      <c r="P50" s="54" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K50,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
-        <v/>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="P50" s="54"/>
     </row>
     <row r="51">
-      <c r="A51" s="60" t="s">
-        <v>130</v>
+      <c r="A51" s="47" t="s">
+        <v>127</v>
       </c>
       <c r="B51" s="48">
-        <v>3.0</v>
+        <v>1.5</v>
       </c>
       <c r="C51" s="48">
-        <v>2.5</v>
+        <v>4.0</v>
       </c>
       <c r="D51" s="48">
-        <v>2.5</v>
+        <v>5.0</v>
       </c>
       <c r="E51" s="48">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="F51" s="48">
-        <v>0.5</v>
+        <v>0.0</v>
       </c>
       <c r="G51" s="48">
+        <v>5.0</v>
+      </c>
+      <c r="H51" s="48">
+        <v>1.0</v>
+      </c>
+      <c r="I51" s="48">
         <v>2.0</v>
       </c>
-      <c r="H51" s="48">
-        <v>2.0</v>
-      </c>
-      <c r="I51" s="48">
-        <v>4.0</v>
-      </c>
       <c r="J51" s="49" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="K51" s="50">
-        <v>19.5</v>
+        <v>20.5</v>
       </c>
       <c r="L51" s="51">
-        <v>19.0</v>
+        <v>20.25</v>
       </c>
       <c r="M51" s="52">
         <f t="shared" si="1"/>
-        <v>0.475</v>
+        <v>0.50625</v>
       </c>
       <c r="N51" s="53" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="P51" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K51,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3616,93 +3616,96 @@
     </row>
     <row r="52">
       <c r="A52" s="60" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B52" s="48">
+        <v>0.0</v>
+      </c>
+      <c r="C52" s="48">
         <v>1.5</v>
       </c>
-      <c r="C52" s="48">
-        <v>0.5</v>
-      </c>
       <c r="D52" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="E52" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="F52" s="48">
+        <v>4.5</v>
+      </c>
+      <c r="G52" s="48">
         <v>2.0</v>
       </c>
-      <c r="E52" s="48">
-        <v>1.5</v>
-      </c>
-      <c r="F52" s="48">
+      <c r="H52" s="48">
         <v>2.0</v>
-      </c>
-      <c r="G52" s="48">
-        <v>3.5</v>
-      </c>
-      <c r="H52" s="48">
-        <v>1.5</v>
       </c>
       <c r="I52" s="48">
         <v>3.5</v>
       </c>
       <c r="J52" s="49" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K52" s="50">
-        <v>16.0</v>
+        <v>19.5</v>
       </c>
       <c r="L52" s="51">
-        <v>15.75</v>
+        <v>19.25</v>
       </c>
       <c r="M52" s="52">
         <f t="shared" si="1"/>
-        <v>0.39375</v>
+        <v>0.48125</v>
       </c>
       <c r="N52" s="53" t="s">
-        <v>101</v>
-      </c>
-      <c r="P52" s="54"/>
+        <v>119</v>
+      </c>
+      <c r="P52" s="54" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K52,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="60" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B53" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="C53" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="D53" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="E53" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="F53" s="48">
         <v>0.5</v>
-      </c>
-      <c r="C53" s="48">
-        <v>3.0</v>
-      </c>
-      <c r="D53" s="48">
-        <v>3.5</v>
-      </c>
-      <c r="E53" s="48">
-        <v>2.5</v>
-      </c>
-      <c r="F53" s="48">
-        <v>0.0</v>
       </c>
       <c r="G53" s="48">
         <v>2.0</v>
       </c>
       <c r="H53" s="48">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="I53" s="48">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="J53" s="49" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K53" s="50">
-        <v>15.5</v>
+        <v>19.5</v>
       </c>
       <c r="L53" s="51">
-        <v>15.25</v>
+        <v>19.0</v>
       </c>
       <c r="M53" s="52">
         <f t="shared" si="1"/>
-        <v>0.38125</v>
+        <v>0.475</v>
       </c>
       <c r="N53" s="53" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="P53" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K53,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3711,44 +3714,44 @@
     </row>
     <row r="54">
       <c r="A54" s="60" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B54" s="48">
         <v>1.5</v>
       </c>
       <c r="C54" s="48">
-        <v>2.5</v>
+        <v>0.5</v>
       </c>
       <c r="D54" s="48">
         <v>2.0</v>
       </c>
       <c r="E54" s="48">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="F54" s="48">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="G54" s="48">
-        <v>3.0</v>
+        <v>3.5</v>
       </c>
       <c r="H54" s="48">
-        <v>1.0</v>
+        <v>1.5</v>
       </c>
       <c r="I54" s="48">
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
       <c r="J54" s="49" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="K54" s="50">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
       <c r="L54" s="51">
-        <v>15.0</v>
+        <v>15.75</v>
       </c>
       <c r="M54" s="52">
         <f t="shared" si="1"/>
-        <v>0.375</v>
+        <v>0.39375</v>
       </c>
       <c r="N54" s="53" t="s">
         <v>101</v>
@@ -3756,164 +3759,243 @@
       <c r="P54" s="54"/>
     </row>
     <row r="55">
-      <c r="A55" s="47" t="s">
-        <v>138</v>
+      <c r="A55" s="60" t="s">
+        <v>136</v>
       </c>
       <c r="B55" s="48">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="C55" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="D55" s="48">
+        <v>3.5</v>
+      </c>
+      <c r="E55" s="48">
         <v>2.5</v>
       </c>
-      <c r="D55" s="48">
-        <v>2.5</v>
-      </c>
-      <c r="E55" s="48">
-        <v>0.5</v>
-      </c>
       <c r="F55" s="48">
-        <v>2.5</v>
+        <v>0.0</v>
       </c>
       <c r="G55" s="48">
-        <v>2.5</v>
+        <v>2.0</v>
       </c>
       <c r="H55" s="48">
-        <v>1.5</v>
+        <v>1.0</v>
       </c>
       <c r="I55" s="48">
-        <v>1.5</v>
+        <v>3.0</v>
       </c>
       <c r="J55" s="49" t="s">
         <v>137</v>
       </c>
       <c r="K55" s="50">
-        <v>15.0</v>
+        <v>15.5</v>
       </c>
       <c r="L55" s="51">
-        <v>15.0</v>
+        <v>15.25</v>
       </c>
       <c r="M55" s="52">
         <f t="shared" si="1"/>
-        <v>0.375</v>
+        <v>0.38125</v>
       </c>
       <c r="N55" s="53" t="s">
-        <v>87</v>
-      </c>
-      <c r="P55" s="54"/>
+        <v>129</v>
+      </c>
+      <c r="P55" s="54" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K55,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="60" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B56" s="48">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="C56" s="48">
-        <v>0.0</v>
+        <v>2.5</v>
       </c>
       <c r="D56" s="48">
-        <v>0.5</v>
+        <v>2.0</v>
       </c>
       <c r="E56" s="48">
         <v>0.5</v>
       </c>
       <c r="F56" s="48">
-        <v>0.0</v>
+        <v>3.0</v>
       </c>
       <c r="G56" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="H56" s="48">
         <v>1.0</v>
       </c>
-      <c r="H56" s="48">
-        <v>0.5</v>
-      </c>
       <c r="I56" s="48">
-        <v>3.0</v>
+        <v>1.5</v>
       </c>
       <c r="J56" s="49" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K56" s="50">
-        <v>6.5</v>
+        <v>15.0</v>
       </c>
       <c r="L56" s="51">
-        <v>6.25</v>
+        <v>15.0</v>
       </c>
       <c r="M56" s="52">
         <f t="shared" si="1"/>
-        <v>0.15625</v>
+        <v>0.375</v>
       </c>
       <c r="N56" s="53" t="s">
-        <v>127</v>
-      </c>
-      <c r="P56" s="54" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K56,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
-        <v/>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="P56" s="54"/>
     </row>
     <row r="57">
-      <c r="A57" s="61" t="s">
-        <v>141</v>
-      </c>
-      <c r="B57" s="62">
-        <v>1.0</v>
-      </c>
-      <c r="C57" s="62">
-        <v>0.0</v>
-      </c>
-      <c r="D57" s="62">
+      <c r="A57" s="47" t="s">
+        <v>140</v>
+      </c>
+      <c r="B57" s="48">
+        <v>1.5</v>
+      </c>
+      <c r="C57" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="D57" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="E57" s="48">
         <v>0.5</v>
       </c>
-      <c r="E57" s="62">
-        <v>0.5</v>
-      </c>
-      <c r="F57" s="62">
-        <v>0.0</v>
-      </c>
-      <c r="G57" s="62">
-        <v>0.0</v>
-      </c>
-      <c r="H57" s="62">
-        <v>0.5</v>
-      </c>
-      <c r="I57" s="62">
-        <v>0.5</v>
-      </c>
-      <c r="J57" s="63" t="s">
-        <v>142</v>
-      </c>
-      <c r="K57" s="64">
-        <v>3.5</v>
-      </c>
-      <c r="L57" s="65">
-        <v>3.25</v>
+      <c r="F57" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="G57" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="H57" s="48">
+        <v>1.5</v>
+      </c>
+      <c r="I57" s="48">
+        <v>1.5</v>
+      </c>
+      <c r="J57" s="49" t="s">
+        <v>139</v>
+      </c>
+      <c r="K57" s="50">
+        <v>15.0</v>
+      </c>
+      <c r="L57" s="51">
+        <v>15.0</v>
       </c>
       <c r="M57" s="52">
         <f t="shared" si="1"/>
-        <v>0.08125</v>
+        <v>0.375</v>
       </c>
       <c r="N57" s="53" t="s">
-        <v>127</v>
-      </c>
-      <c r="P57" s="54" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K57,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
+        <v>87</v>
+      </c>
+      <c r="P57" s="54"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="60" t="s">
+        <v>141</v>
+      </c>
+      <c r="B58" s="48">
+        <v>0.5</v>
+      </c>
+      <c r="C58" s="48">
+        <v>0.0</v>
+      </c>
+      <c r="D58" s="48">
+        <v>0.5</v>
+      </c>
+      <c r="E58" s="48">
+        <v>0.5</v>
+      </c>
+      <c r="F58" s="48">
+        <v>0.0</v>
+      </c>
+      <c r="G58" s="48">
+        <v>1.0</v>
+      </c>
+      <c r="H58" s="48">
+        <v>0.5</v>
+      </c>
+      <c r="I58" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="J58" s="49" t="s">
+        <v>142</v>
+      </c>
+      <c r="K58" s="58">
+        <v>6.0</v>
+      </c>
+      <c r="L58" s="59">
+        <v>5.75</v>
+      </c>
+      <c r="M58" s="52">
+        <f t="shared" si="1"/>
+        <v>0.14375</v>
+      </c>
+      <c r="N58" s="53" t="s">
+        <v>129</v>
+      </c>
+      <c r="P58" s="54" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K58,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
         <v/>
       </c>
     </row>
-    <row r="58">
-      <c r="J58" s="66"/>
-      <c r="K58" s="67"/>
-      <c r="L58" s="68"/>
-      <c r="M58" s="69"/>
-      <c r="N58" s="70"/>
-      <c r="P58" s="71"/>
-    </row>
     <row r="59">
-      <c r="J59" s="66"/>
-      <c r="K59" s="67"/>
-      <c r="L59" s="68"/>
-      <c r="M59" s="69"/>
-      <c r="N59" s="70"/>
-      <c r="P59" s="71"/>
+      <c r="A59" s="61" t="s">
+        <v>143</v>
+      </c>
+      <c r="B59" s="62">
+        <v>1.0</v>
+      </c>
+      <c r="C59" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="D59" s="62">
+        <v>0.5</v>
+      </c>
+      <c r="E59" s="62">
+        <v>0.5</v>
+      </c>
+      <c r="F59" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="G59" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="H59" s="62">
+        <v>0.5</v>
+      </c>
+      <c r="I59" s="62">
+        <v>0.5</v>
+      </c>
+      <c r="J59" s="63" t="s">
+        <v>144</v>
+      </c>
+      <c r="K59" s="64">
+        <v>3.0</v>
+      </c>
+      <c r="L59" s="65">
+        <v>2.75</v>
+      </c>
+      <c r="M59" s="52">
+        <f t="shared" si="1"/>
+        <v>0.06875</v>
+      </c>
+      <c r="N59" s="53" t="s">
+        <v>129</v>
+      </c>
+      <c r="P59" s="54" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K59,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="J60" s="66"/>
@@ -11531,19 +11613,35 @@
       <c r="N1011" s="70"/>
       <c r="P1011" s="71"/>
     </row>
+    <row r="1012">
+      <c r="J1012" s="66"/>
+      <c r="K1012" s="67"/>
+      <c r="L1012" s="68"/>
+      <c r="M1012" s="69"/>
+      <c r="N1012" s="70"/>
+      <c r="P1012" s="71"/>
+    </row>
+    <row r="1013">
+      <c r="J1013" s="66"/>
+      <c r="K1013" s="67"/>
+      <c r="L1013" s="68"/>
+      <c r="M1013" s="69"/>
+      <c r="N1013" s="70"/>
+      <c r="P1013" s="71"/>
+    </row>
   </sheetData>
-  <autoFilter ref="$A$7:$P$57">
-    <sortState ref="A7:P57">
-      <sortCondition descending="1" ref="L7:L57"/>
-      <sortCondition descending="1" ref="P7:P57"/>
-      <sortCondition descending="1" ref="I7:I57"/>
-      <sortCondition descending="1" ref="F7:F57"/>
-      <sortCondition descending="1" ref="H7:H57"/>
-      <sortCondition descending="1" ref="G7:G57"/>
-      <sortCondition descending="1" ref="E7:E57"/>
-      <sortCondition descending="1" ref="D7:D57"/>
-      <sortCondition descending="1" ref="C7:C57"/>
-      <sortCondition descending="1" ref="B7:B57"/>
+  <autoFilter ref="$A$7:$P$59">
+    <sortState ref="A7:P59">
+      <sortCondition descending="1" ref="L7:L59"/>
+      <sortCondition descending="1" ref="P7:P59"/>
+      <sortCondition descending="1" ref="I7:I59"/>
+      <sortCondition descending="1" ref="F7:F59"/>
+      <sortCondition descending="1" ref="H7:H59"/>
+      <sortCondition descending="1" ref="G7:G59"/>
+      <sortCondition descending="1" ref="E7:E59"/>
+      <sortCondition descending="1" ref="D7:D59"/>
+      <sortCondition descending="1" ref="C7:C59"/>
+      <sortCondition descending="1" ref="B7:B59"/>
     </sortState>
   </autoFilter>
   <mergeCells count="3">
@@ -11551,7 +11649,7 @@
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="G4:H4"/>
   </mergeCells>
-  <conditionalFormatting sqref="B8:I57">
+  <conditionalFormatting sqref="B8:I59">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -11564,7 +11662,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="N8:N57">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="N8:N59">
       <formula1>"100 %,75 %,50 %,25 %,0 %,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Plot the round v4.14 (Against the Storm + Frostpunk)
</commit_message>
<xml_diff>
--- a/assets/ledger.xlsx
+++ b/assets/ledger.xlsx
@@ -6,14 +6,14 @@
     <sheet state="visible" name="ledger" sheetId="1" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">ledger!$A$7:$P$59</definedName>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">ledger!$A$7:$P$61</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="148">
   <si>
     <t>Civ-likeness Rating System</t>
   </si>
@@ -405,19 +405,28 @@
     <t>19.5/1.0</t>
   </si>
   <si>
+    <t>Against the Storm (2023–current, +2 DLC)</t>
+  </si>
+  <si>
+    <t>17.0/2.5</t>
+  </si>
+  <si>
+    <t>Football Manager 26 (final)</t>
+  </si>
+  <si>
+    <t>13.0/6.5</t>
+  </si>
+  <si>
+    <t>Frostpunk (2018–20, +Season Pass)</t>
+  </si>
+  <si>
+    <t>16.0/3.5</t>
+  </si>
+  <si>
+    <t>XCOM 2 (2017, WotC)</t>
+  </si>
+  <si>
     <t>N/A</t>
-  </si>
-  <si>
-    <t>Football Manager 26 (final)</t>
-  </si>
-  <si>
-    <t>13.0/6.5</t>
-  </si>
-  <si>
-    <t>XCOM 2 (2017, WotC)</t>
-  </si>
-  <si>
-    <t>17.0/2.5</t>
   </si>
   <si>
     <t>Fantasy General (1996, +Island Challenge)</t>
@@ -1526,7 +1535,7 @@
         <v>40.0</v>
       </c>
       <c r="M8" s="52">
-        <f t="shared" ref="M8:M59" si="1">L8/40</f>
+        <f t="shared" ref="M8:M61" si="1">L8/40</f>
         <v>1</v>
       </c>
       <c r="N8" s="53" t="s">
@@ -3507,7 +3516,7 @@
       <c r="K49" s="50">
         <v>24.0</v>
       </c>
-      <c r="L49" s="56">
+      <c r="L49" s="51">
         <v>23.75</v>
       </c>
       <c r="M49" s="52">
@@ -3607,7 +3616,7 @@
         <v>0.50625</v>
       </c>
       <c r="N51" s="53" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="P51" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K51,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3615,72 +3624,69 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="60" t="s">
-        <v>130</v>
+      <c r="A52" s="47" t="s">
+        <v>129</v>
       </c>
       <c r="B52" s="48">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="C52" s="48">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="D52" s="48">
+        <v>4.5</v>
+      </c>
+      <c r="E52" s="48">
+        <v>2.0</v>
+      </c>
+      <c r="F52" s="48">
+        <v>0.5</v>
+      </c>
+      <c r="G52" s="48">
         <v>3.0</v>
-      </c>
-      <c r="E52" s="48">
-        <v>3.0</v>
-      </c>
-      <c r="F52" s="48">
-        <v>4.5</v>
-      </c>
-      <c r="G52" s="48">
-        <v>2.0</v>
       </c>
       <c r="H52" s="48">
         <v>2.0</v>
       </c>
       <c r="I52" s="48">
-        <v>3.5</v>
+        <v>3.0</v>
       </c>
       <c r="J52" s="49" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="K52" s="50">
         <v>19.5</v>
       </c>
       <c r="L52" s="51">
-        <v>19.25</v>
+        <v>19.5</v>
       </c>
       <c r="M52" s="52">
         <f t="shared" si="1"/>
-        <v>0.48125</v>
+        <v>0.4875</v>
       </c>
       <c r="N52" s="53" t="s">
         <v>119</v>
       </c>
-      <c r="P52" s="54" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K52,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
-        <v/>
-      </c>
+      <c r="P52" s="54"/>
     </row>
     <row r="53">
       <c r="A53" s="60" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B53" s="48">
+        <v>0.0</v>
+      </c>
+      <c r="C53" s="48">
+        <v>1.5</v>
+      </c>
+      <c r="D53" s="48">
         <v>3.0</v>
-      </c>
-      <c r="C53" s="48">
-        <v>2.5</v>
-      </c>
-      <c r="D53" s="48">
-        <v>2.5</v>
       </c>
       <c r="E53" s="48">
         <v>3.0</v>
       </c>
       <c r="F53" s="48">
-        <v>0.5</v>
+        <v>4.5</v>
       </c>
       <c r="G53" s="48">
         <v>2.0</v>
@@ -3689,23 +3695,23 @@
         <v>2.0</v>
       </c>
       <c r="I53" s="48">
-        <v>4.0</v>
+        <v>3.5</v>
       </c>
       <c r="J53" s="49" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K53" s="50">
         <v>19.5</v>
       </c>
       <c r="L53" s="51">
-        <v>19.0</v>
+        <v>19.25</v>
       </c>
       <c r="M53" s="52">
         <f t="shared" si="1"/>
-        <v>0.475</v>
+        <v>0.48125</v>
       </c>
       <c r="N53" s="53" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="P53" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K53,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3713,94 +3719,94 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="60" t="s">
-        <v>134</v>
+      <c r="A54" s="47" t="s">
+        <v>133</v>
       </c>
       <c r="B54" s="48">
         <v>1.5</v>
       </c>
       <c r="C54" s="48">
+        <v>2.0</v>
+      </c>
+      <c r="D54" s="48">
+        <v>4.0</v>
+      </c>
+      <c r="E54" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="F54" s="48">
         <v>0.5</v>
       </c>
-      <c r="D54" s="48">
-        <v>2.0</v>
-      </c>
-      <c r="E54" s="48">
-        <v>1.5</v>
-      </c>
-      <c r="F54" s="48">
-        <v>2.0</v>
-      </c>
       <c r="G54" s="48">
-        <v>3.5</v>
+        <v>3.0</v>
       </c>
       <c r="H54" s="48">
-        <v>1.5</v>
+        <v>3.0</v>
       </c>
       <c r="I54" s="48">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="J54" s="49" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="K54" s="50">
-        <v>16.0</v>
+        <v>19.5</v>
       </c>
       <c r="L54" s="51">
-        <v>15.75</v>
+        <v>19.25</v>
       </c>
       <c r="M54" s="52">
         <f t="shared" si="1"/>
-        <v>0.39375</v>
+        <v>0.48125</v>
       </c>
       <c r="N54" s="53" t="s">
-        <v>101</v>
+        <v>119</v>
       </c>
       <c r="P54" s="54"/>
     </row>
     <row r="55">
       <c r="A55" s="60" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B55" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="C55" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="D55" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="E55" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="F55" s="48">
         <v>0.5</v>
-      </c>
-      <c r="C55" s="48">
-        <v>3.0</v>
-      </c>
-      <c r="D55" s="48">
-        <v>3.5</v>
-      </c>
-      <c r="E55" s="48">
-        <v>2.5</v>
-      </c>
-      <c r="F55" s="48">
-        <v>0.0</v>
       </c>
       <c r="G55" s="48">
         <v>2.0</v>
       </c>
       <c r="H55" s="48">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="I55" s="48">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="J55" s="49" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="K55" s="50">
-        <v>15.5</v>
+        <v>19.5</v>
       </c>
       <c r="L55" s="51">
-        <v>15.25</v>
+        <v>19.0</v>
       </c>
       <c r="M55" s="52">
         <f t="shared" si="1"/>
-        <v>0.38125</v>
+        <v>0.475</v>
       </c>
       <c r="N55" s="53" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="P55" s="54" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K55,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
@@ -3809,44 +3815,44 @@
     </row>
     <row r="56">
       <c r="A56" s="60" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B56" s="48">
         <v>1.5</v>
       </c>
       <c r="C56" s="48">
-        <v>2.5</v>
+        <v>0.5</v>
       </c>
       <c r="D56" s="48">
         <v>2.0</v>
       </c>
       <c r="E56" s="48">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="F56" s="48">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="G56" s="48">
-        <v>3.0</v>
+        <v>3.5</v>
       </c>
       <c r="H56" s="48">
-        <v>1.0</v>
+        <v>1.5</v>
       </c>
       <c r="I56" s="48">
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
       <c r="J56" s="49" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K56" s="50">
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
       <c r="L56" s="51">
-        <v>15.0</v>
+        <v>15.75</v>
       </c>
       <c r="M56" s="52">
         <f t="shared" si="1"/>
-        <v>0.375</v>
+        <v>0.39375</v>
       </c>
       <c r="N56" s="53" t="s">
         <v>101</v>
@@ -3854,164 +3860,243 @@
       <c r="P56" s="54"/>
     </row>
     <row r="57">
-      <c r="A57" s="47" t="s">
+      <c r="A57" s="60" t="s">
+        <v>139</v>
+      </c>
+      <c r="B57" s="48">
+        <v>0.5</v>
+      </c>
+      <c r="C57" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="D57" s="48">
+        <v>3.5</v>
+      </c>
+      <c r="E57" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="F57" s="48">
+        <v>0.0</v>
+      </c>
+      <c r="G57" s="48">
+        <v>2.0</v>
+      </c>
+      <c r="H57" s="48">
+        <v>1.0</v>
+      </c>
+      <c r="I57" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="J57" s="49" t="s">
         <v>140</v>
       </c>
-      <c r="B57" s="48">
-        <v>1.5</v>
-      </c>
-      <c r="C57" s="48">
-        <v>2.5</v>
-      </c>
-      <c r="D57" s="48">
-        <v>2.5</v>
-      </c>
-      <c r="E57" s="48">
-        <v>0.5</v>
-      </c>
-      <c r="F57" s="48">
-        <v>2.5</v>
-      </c>
-      <c r="G57" s="48">
-        <v>2.5</v>
-      </c>
-      <c r="H57" s="48">
-        <v>1.5</v>
-      </c>
-      <c r="I57" s="48">
-        <v>1.5</v>
-      </c>
-      <c r="J57" s="49" t="s">
-        <v>139</v>
-      </c>
       <c r="K57" s="50">
-        <v>15.0</v>
+        <v>15.5</v>
       </c>
       <c r="L57" s="51">
-        <v>15.0</v>
+        <v>15.25</v>
       </c>
       <c r="M57" s="52">
         <f t="shared" si="1"/>
-        <v>0.375</v>
+        <v>0.38125</v>
       </c>
       <c r="N57" s="53" t="s">
-        <v>87</v>
-      </c>
-      <c r="P57" s="54"/>
+        <v>136</v>
+      </c>
+      <c r="P57" s="54" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K57,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="60" t="s">
         <v>141</v>
       </c>
       <c r="B58" s="48">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="C58" s="48">
-        <v>0.0</v>
+        <v>2.5</v>
       </c>
       <c r="D58" s="48">
-        <v>0.5</v>
+        <v>2.0</v>
       </c>
       <c r="E58" s="48">
         <v>0.5</v>
       </c>
       <c r="F58" s="48">
-        <v>0.0</v>
+        <v>3.0</v>
       </c>
       <c r="G58" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="H58" s="48">
         <v>1.0</v>
       </c>
-      <c r="H58" s="48">
-        <v>0.5</v>
-      </c>
       <c r="I58" s="48">
-        <v>3.0</v>
+        <v>1.5</v>
       </c>
       <c r="J58" s="49" t="s">
         <v>142</v>
       </c>
-      <c r="K58" s="58">
-        <v>6.0</v>
-      </c>
-      <c r="L58" s="59">
-        <v>5.75</v>
+      <c r="K58" s="50">
+        <v>15.0</v>
+      </c>
+      <c r="L58" s="51">
+        <v>15.0</v>
       </c>
       <c r="M58" s="52">
         <f t="shared" si="1"/>
-        <v>0.14375</v>
+        <v>0.375</v>
       </c>
       <c r="N58" s="53" t="s">
-        <v>129</v>
-      </c>
-      <c r="P58" s="54" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K58,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
-        <v/>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="P58" s="54"/>
     </row>
     <row r="59">
-      <c r="A59" s="61" t="s">
+      <c r="A59" s="47" t="s">
         <v>143</v>
       </c>
-      <c r="B59" s="62">
-        <v>1.0</v>
-      </c>
-      <c r="C59" s="62">
-        <v>0.0</v>
-      </c>
-      <c r="D59" s="62">
+      <c r="B59" s="48">
+        <v>1.5</v>
+      </c>
+      <c r="C59" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="D59" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="E59" s="48">
         <v>0.5</v>
       </c>
-      <c r="E59" s="62">
-        <v>0.5</v>
-      </c>
-      <c r="F59" s="62">
-        <v>0.0</v>
-      </c>
-      <c r="G59" s="62">
-        <v>0.0</v>
-      </c>
-      <c r="H59" s="62">
-        <v>0.5</v>
-      </c>
-      <c r="I59" s="62">
-        <v>0.5</v>
-      </c>
-      <c r="J59" s="63" t="s">
-        <v>144</v>
-      </c>
-      <c r="K59" s="64">
-        <v>3.0</v>
-      </c>
-      <c r="L59" s="65">
-        <v>2.75</v>
+      <c r="F59" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="G59" s="48">
+        <v>2.5</v>
+      </c>
+      <c r="H59" s="48">
+        <v>1.5</v>
+      </c>
+      <c r="I59" s="48">
+        <v>1.5</v>
+      </c>
+      <c r="J59" s="49" t="s">
+        <v>142</v>
+      </c>
+      <c r="K59" s="50">
+        <v>15.0</v>
+      </c>
+      <c r="L59" s="51">
+        <v>15.0</v>
       </c>
       <c r="M59" s="52">
         <f t="shared" si="1"/>
+        <v>0.375</v>
+      </c>
+      <c r="N59" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="P59" s="54"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="60" t="s">
+        <v>144</v>
+      </c>
+      <c r="B60" s="48">
+        <v>0.5</v>
+      </c>
+      <c r="C60" s="48">
+        <v>0.0</v>
+      </c>
+      <c r="D60" s="48">
+        <v>0.5</v>
+      </c>
+      <c r="E60" s="48">
+        <v>0.5</v>
+      </c>
+      <c r="F60" s="48">
+        <v>0.0</v>
+      </c>
+      <c r="G60" s="48">
+        <v>1.0</v>
+      </c>
+      <c r="H60" s="48">
+        <v>0.5</v>
+      </c>
+      <c r="I60" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="J60" s="49" t="s">
+        <v>145</v>
+      </c>
+      <c r="K60" s="58">
+        <v>6.0</v>
+      </c>
+      <c r="L60" s="59">
+        <v>5.75</v>
+      </c>
+      <c r="M60" s="52">
+        <f t="shared" si="1"/>
+        <v>0.14375</v>
+      </c>
+      <c r="N60" s="53" t="s">
+        <v>136</v>
+      </c>
+      <c r="P60" s="54" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K60,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="61" t="s">
+        <v>146</v>
+      </c>
+      <c r="B61" s="62">
+        <v>1.0</v>
+      </c>
+      <c r="C61" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="D61" s="62">
+        <v>0.5</v>
+      </c>
+      <c r="E61" s="62">
+        <v>0.5</v>
+      </c>
+      <c r="F61" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="G61" s="62">
+        <v>0.0</v>
+      </c>
+      <c r="H61" s="62">
+        <v>0.5</v>
+      </c>
+      <c r="I61" s="62">
+        <v>0.5</v>
+      </c>
+      <c r="J61" s="63" t="s">
+        <v>147</v>
+      </c>
+      <c r="K61" s="64">
+        <v>3.0</v>
+      </c>
+      <c r="L61" s="65">
+        <v>2.75</v>
+      </c>
+      <c r="M61" s="52">
+        <f t="shared" si="1"/>
         <v>0.06875</v>
       </c>
-      <c r="N59" s="53" t="s">
-        <v>129</v>
-      </c>
-      <c r="P59" s="54" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K59,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
+      <c r="N61" s="53" t="s">
+        <v>136</v>
+      </c>
+      <c r="P61" s="54" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("IFERROR(VALUE(REGEXEXTRACT(K61,""^[0-9]+(?:\.[0-9]+)?"")),)"),"")</f>
         <v/>
       </c>
-    </row>
-    <row r="60">
-      <c r="J60" s="66"/>
-      <c r="K60" s="67"/>
-      <c r="L60" s="68"/>
-      <c r="M60" s="69"/>
-      <c r="N60" s="70"/>
-      <c r="P60" s="71"/>
-    </row>
-    <row r="61">
-      <c r="J61" s="66"/>
-      <c r="K61" s="67"/>
-      <c r="L61" s="68"/>
-      <c r="M61" s="69"/>
-      <c r="N61" s="70"/>
-      <c r="P61" s="71"/>
     </row>
     <row r="62">
       <c r="J62" s="66"/>
@@ -11629,19 +11714,35 @@
       <c r="N1013" s="70"/>
       <c r="P1013" s="71"/>
     </row>
+    <row r="1014">
+      <c r="J1014" s="66"/>
+      <c r="K1014" s="67"/>
+      <c r="L1014" s="68"/>
+      <c r="M1014" s="69"/>
+      <c r="N1014" s="70"/>
+      <c r="P1014" s="71"/>
+    </row>
+    <row r="1015">
+      <c r="J1015" s="66"/>
+      <c r="K1015" s="67"/>
+      <c r="L1015" s="68"/>
+      <c r="M1015" s="69"/>
+      <c r="N1015" s="70"/>
+      <c r="P1015" s="71"/>
+    </row>
   </sheetData>
-  <autoFilter ref="$A$7:$P$59">
-    <sortState ref="A7:P59">
-      <sortCondition descending="1" ref="L7:L59"/>
-      <sortCondition descending="1" ref="P7:P59"/>
-      <sortCondition descending="1" ref="I7:I59"/>
-      <sortCondition descending="1" ref="F7:F59"/>
-      <sortCondition descending="1" ref="H7:H59"/>
-      <sortCondition descending="1" ref="G7:G59"/>
-      <sortCondition descending="1" ref="E7:E59"/>
-      <sortCondition descending="1" ref="D7:D59"/>
-      <sortCondition descending="1" ref="C7:C59"/>
-      <sortCondition descending="1" ref="B7:B59"/>
+  <autoFilter ref="$A$7:$P$61">
+    <sortState ref="A7:P61">
+      <sortCondition descending="1" ref="L7:L61"/>
+      <sortCondition descending="1" ref="P7:P61"/>
+      <sortCondition descending="1" ref="I7:I61"/>
+      <sortCondition descending="1" ref="F7:F61"/>
+      <sortCondition descending="1" ref="H7:H61"/>
+      <sortCondition descending="1" ref="G7:G61"/>
+      <sortCondition descending="1" ref="E7:E61"/>
+      <sortCondition descending="1" ref="D7:D61"/>
+      <sortCondition descending="1" ref="C7:C61"/>
+      <sortCondition descending="1" ref="B7:B61"/>
     </sortState>
   </autoFilter>
   <mergeCells count="3">
@@ -11649,7 +11750,7 @@
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="G4:H4"/>
   </mergeCells>
-  <conditionalFormatting sqref="B8:I59">
+  <conditionalFormatting sqref="B8:I61">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -11662,7 +11763,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="N8:N59">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="N8:N61">
       <formula1>"100 %,75 %,50 %,25 %,0 %,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>